<commit_message>
Add new items delivery and spare-parts placeholder export
</commit_message>
<xml_diff>
--- a/final_elitech_and_teh_delivery_2026-04-27/pictures_for_bitrix_import.xlsx
+++ b/final_elitech_and_teh_delivery_2026-04-27/pictures_for_bitrix_import.xlsx
@@ -456,11 +456,7 @@
           <t>/upload/vvm_images/import_images/TPS728-B/preview.webp</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TPS728-B/nan</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -473,11 +469,7 @@
           <t>/upload/vvm_images/import_images/204458/preview.webp</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204458/nan</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -492,7 +484,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205819/gallery_01.webp|/upload/vvm_images/import_images/205819/gallery_02.webp|/upload/vvm_images/import_images/205819/gallery_03.webp|/upload/vvm_images/import_images/205819/gallery_04.webp|/upload/vvm_images/import_images/205819/gallery_05.webp|/upload/vvm_images/import_images/205819/gallery_06.webp</t>
+          <t>/upload/vvm_images/import_images/205819/gallery_01.webp;/upload/vvm_images/import_images/205819/gallery_02.webp;/upload/vvm_images/import_images/205819/gallery_03.webp;/upload/vvm_images/import_images/205819/gallery_04.webp;/upload/vvm_images/import_images/205819/gallery_05.webp;/upload/vvm_images/import_images/205819/gallery_06.webp</t>
         </is>
       </c>
     </row>
@@ -509,7 +501,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205859/gallery_01.webp|/upload/vvm_images/import_images/205859/gallery_02.webp|/upload/vvm_images/import_images/205859/gallery_03.webp|/upload/vvm_images/import_images/205859/gallery_04.webp|/upload/vvm_images/import_images/205859/gallery_05.webp|/upload/vvm_images/import_images/205859/gallery_06.webp</t>
+          <t>/upload/vvm_images/import_images/205859/gallery_01.webp;/upload/vvm_images/import_images/205859/gallery_02.webp;/upload/vvm_images/import_images/205859/gallery_03.webp;/upload/vvm_images/import_images/205859/gallery_04.webp;/upload/vvm_images/import_images/205859/gallery_05.webp;/upload/vvm_images/import_images/205859/gallery_06.webp</t>
         </is>
       </c>
     </row>
@@ -526,7 +518,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205862/gallery_01.webp|/upload/vvm_images/import_images/205862/gallery_02.webp|/upload/vvm_images/import_images/205862/gallery_03.webp|/upload/vvm_images/import_images/205862/gallery_04.webp|/upload/vvm_images/import_images/205862/gallery_05.webp|/upload/vvm_images/import_images/205862/gallery_06.webp</t>
+          <t>/upload/vvm_images/import_images/205862/gallery_01.webp;/upload/vvm_images/import_images/205862/gallery_02.webp;/upload/vvm_images/import_images/205862/gallery_03.webp;/upload/vvm_images/import_images/205862/gallery_04.webp;/upload/vvm_images/import_images/205862/gallery_05.webp;/upload/vvm_images/import_images/205862/gallery_06.webp</t>
         </is>
       </c>
     </row>
@@ -541,11 +533,7 @@
           <t>/upload/vvm_images/import_images/215218/preview.webp</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215218/nan</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -558,11 +546,7 @@
           <t>/upload/vvm_images/import_images/215227/preview.webp</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215227/nan</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -575,11 +559,7 @@
           <t>/upload/vvm_images/import_images/215233/preview.webp</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215233/nan</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -592,11 +572,7 @@
           <t>/upload/vvm_images/import_images/215219/preview.webp</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215219/nan</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -609,11 +585,7 @@
           <t>/upload/vvm_images/import_images/215220/preview.webp</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215220/nan</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -626,11 +598,7 @@
           <t>/upload/vvm_images/import_images/215229/preview.webp</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215229/nan</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -643,11 +611,7 @@
           <t>/upload/vvm_images/import_images/215236/preview.webp</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215236/nan</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -660,11 +624,7 @@
           <t>/upload/vvm_images/import_images/215221/preview.webp</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215221/nan</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -677,11 +637,7 @@
           <t>/upload/vvm_images/import_images/215230/preview.webp</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215230/nan</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -696,7 +652,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204252/gallery_01.webp|/upload/vvm_images/import_images/204252/gallery_02.webp|/upload/vvm_images/import_images/204252/gallery_03.webp</t>
+          <t>/upload/vvm_images/import_images/204252/gallery_01.webp;/upload/vvm_images/import_images/204252/gallery_02.webp;/upload/vvm_images/import_images/204252/gallery_03.webp</t>
         </is>
       </c>
     </row>
@@ -713,7 +669,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/215238/gallery_01.webp|/upload/vvm_images/import_images/215238/gallery_02.webp|/upload/vvm_images/import_images/215238/gallery_03.webp</t>
+          <t>/upload/vvm_images/import_images/215238/gallery_01.webp;/upload/vvm_images/import_images/215238/gallery_02.webp;/upload/vvm_images/import_images/215238/gallery_03.webp</t>
         </is>
       </c>
     </row>
@@ -728,11 +684,7 @@
           <t>/upload/vvm_images/import_images/215222/preview.webp</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215222/nan</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -745,11 +697,7 @@
           <t>/upload/vvm_images/import_images/215231/preview.webp</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215231/nan</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -762,11 +710,7 @@
           <t>/upload/vvm_images/import_images/215235/preview.webp</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215235/nan</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -779,11 +723,7 @@
           <t>/upload/vvm_images/import_images/215223/preview.webp</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215223/nan</t>
-        </is>
-      </c>
+      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -796,11 +736,7 @@
           <t>/upload/vvm_images/import_images/215232/preview.webp</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215232/nan</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -815,7 +751,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204251/gallery_01.webp|/upload/vvm_images/import_images/204251/gallery_02.webp</t>
+          <t>/upload/vvm_images/import_images/204251/gallery_01.webp;/upload/vvm_images/import_images/204251/gallery_02.webp</t>
         </is>
       </c>
     </row>
@@ -832,7 +768,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/215237/gallery_01.webp|/upload/vvm_images/import_images/215237/gallery_02.webp</t>
+          <t>/upload/vvm_images/import_images/215237/gallery_01.webp;/upload/vvm_images/import_images/215237/gallery_02.webp</t>
         </is>
       </c>
     </row>
@@ -847,11 +783,7 @@
           <t>/upload/vvm_images/import_images/215226/preview.webp</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215226/nan</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -864,11 +796,7 @@
           <t>/upload/vvm_images/import_images/204201/preview.webp</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204201/nan</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -881,11 +809,7 @@
           <t>/upload/vvm_images/import_images/204200/preview.webp</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204200/nan</t>
-        </is>
-      </c>
+      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -898,11 +822,7 @@
           <t>/upload/vvm_images/import_images/204216/preview.webp</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204216/nan</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -915,11 +835,7 @@
           <t>/upload/vvm_images/import_images/210431/preview.webp</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210431/nan</t>
-        </is>
-      </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -934,7 +850,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205731/gallery_01.webp|/upload/vvm_images/import_images/205731/gallery_02.webp|/upload/vvm_images/import_images/205731/gallery_03.webp|/upload/vvm_images/import_images/205731/gallery_04.webp|/upload/vvm_images/import_images/205731/gallery_05.webp|/upload/vvm_images/import_images/205731/gallery_06.webp|/upload/vvm_images/import_images/205731/gallery_07.webp|/upload/vvm_images/import_images/205731/gallery_08.webp</t>
+          <t>/upload/vvm_images/import_images/205731/gallery_01.webp;/upload/vvm_images/import_images/205731/gallery_02.webp;/upload/vvm_images/import_images/205731/gallery_03.webp;/upload/vvm_images/import_images/205731/gallery_04.webp;/upload/vvm_images/import_images/205731/gallery_05.webp;/upload/vvm_images/import_images/205731/gallery_06.webp;/upload/vvm_images/import_images/205731/gallery_07.webp;/upload/vvm_images/import_images/205731/gallery_08.webp</t>
         </is>
       </c>
     </row>
@@ -949,11 +865,7 @@
           <t>/upload/vvm_images/import_images/210297/preview.webp</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210297/nan</t>
-        </is>
-      </c>
+      <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -966,11 +878,7 @@
           <t>/upload/vvm_images/import_images/205736/preview.webp</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205736/nan</t>
-        </is>
-      </c>
+      <c r="C32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -983,11 +891,7 @@
           <t>/upload/vvm_images/import_images/205746/preview.webp</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205746/nan</t>
-        </is>
-      </c>
+      <c r="C33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1002,7 +906,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210303/gallery_01.webp|/upload/vvm_images/import_images/210303/gallery_02.webp|/upload/vvm_images/import_images/210303/gallery_03.webp|/upload/vvm_images/import_images/210303/gallery_04.webp|/upload/vvm_images/import_images/210303/gallery_05.webp|/upload/vvm_images/import_images/210303/gallery_06.webp|/upload/vvm_images/import_images/210303/gallery_07.webp</t>
+          <t>/upload/vvm_images/import_images/210303/gallery_01.webp;/upload/vvm_images/import_images/210303/gallery_02.webp;/upload/vvm_images/import_images/210303/gallery_03.webp;/upload/vvm_images/import_images/210303/gallery_04.webp;/upload/vvm_images/import_images/210303/gallery_05.webp;/upload/vvm_images/import_images/210303/gallery_06.webp;/upload/vvm_images/import_images/210303/gallery_07.webp</t>
         </is>
       </c>
     </row>
@@ -1019,7 +923,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210304/gallery_01.webp|/upload/vvm_images/import_images/210304/gallery_02.webp|/upload/vvm_images/import_images/210304/gallery_03.webp|/upload/vvm_images/import_images/210304/gallery_04.webp|/upload/vvm_images/import_images/210304/gallery_05.webp|/upload/vvm_images/import_images/210304/gallery_06.webp|/upload/vvm_images/import_images/210304/gallery_07.webp|/upload/vvm_images/import_images/210304/gallery_08.webp|/upload/vvm_images/import_images/210304/gallery_09.webp|/upload/vvm_images/import_images/210304/gallery_10.webp</t>
+          <t>/upload/vvm_images/import_images/210304/gallery_01.webp;/upload/vvm_images/import_images/210304/gallery_02.webp;/upload/vvm_images/import_images/210304/gallery_03.webp;/upload/vvm_images/import_images/210304/gallery_04.webp;/upload/vvm_images/import_images/210304/gallery_05.webp;/upload/vvm_images/import_images/210304/gallery_06.webp;/upload/vvm_images/import_images/210304/gallery_07.webp;/upload/vvm_images/import_images/210304/gallery_08.webp;/upload/vvm_images/import_images/210304/gallery_09.webp;/upload/vvm_images/import_images/210304/gallery_10.webp</t>
         </is>
       </c>
     </row>
@@ -1036,7 +940,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/214178/gallery_01.webp|/upload/vvm_images/import_images/214178/gallery_02.webp|/upload/vvm_images/import_images/214178/gallery_03.webp|/upload/vvm_images/import_images/214178/gallery_04.webp|/upload/vvm_images/import_images/214178/gallery_05.webp|/upload/vvm_images/import_images/214178/gallery_06.webp|/upload/vvm_images/import_images/214178/gallery_07.webp</t>
+          <t>/upload/vvm_images/import_images/214178/gallery_01.webp;/upload/vvm_images/import_images/214178/gallery_02.webp;/upload/vvm_images/import_images/214178/gallery_03.webp;/upload/vvm_images/import_images/214178/gallery_04.webp;/upload/vvm_images/import_images/214178/gallery_05.webp;/upload/vvm_images/import_images/214178/gallery_06.webp;/upload/vvm_images/import_images/214178/gallery_07.webp</t>
         </is>
       </c>
     </row>
@@ -1053,7 +957,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/214180/gallery_01.webp|/upload/vvm_images/import_images/214180/gallery_02.webp|/upload/vvm_images/import_images/214180/gallery_03.webp|/upload/vvm_images/import_images/214180/gallery_04.webp|/upload/vvm_images/import_images/214180/gallery_05.webp|/upload/vvm_images/import_images/214180/gallery_06.webp|/upload/vvm_images/import_images/214180/gallery_07.webp|/upload/vvm_images/import_images/214180/gallery_08.webp|/upload/vvm_images/import_images/214180/gallery_09.webp|/upload/vvm_images/import_images/214180/gallery_10.webp</t>
+          <t>/upload/vvm_images/import_images/214180/gallery_01.webp;/upload/vvm_images/import_images/214180/gallery_02.webp;/upload/vvm_images/import_images/214180/gallery_03.webp;/upload/vvm_images/import_images/214180/gallery_04.webp;/upload/vvm_images/import_images/214180/gallery_05.webp;/upload/vvm_images/import_images/214180/gallery_06.webp;/upload/vvm_images/import_images/214180/gallery_07.webp;/upload/vvm_images/import_images/214180/gallery_08.webp;/upload/vvm_images/import_images/214180/gallery_09.webp;/upload/vvm_images/import_images/214180/gallery_10.webp</t>
         </is>
       </c>
     </row>
@@ -1070,7 +974,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/214184/gallery_01.webp|/upload/vvm_images/import_images/214184/gallery_02.webp|/upload/vvm_images/import_images/214184/gallery_03.webp|/upload/vvm_images/import_images/214184/gallery_04.webp|/upload/vvm_images/import_images/214184/gallery_05.webp|/upload/vvm_images/import_images/214184/gallery_06.webp|/upload/vvm_images/import_images/214184/gallery_07.webp|/upload/vvm_images/import_images/214184/gallery_08.webp|/upload/vvm_images/import_images/214184/gallery_09.webp|/upload/vvm_images/import_images/214184/gallery_10.webp|/upload/vvm_images/import_images/214184/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/214184/gallery_01.webp;/upload/vvm_images/import_images/214184/gallery_02.webp;/upload/vvm_images/import_images/214184/gallery_03.webp;/upload/vvm_images/import_images/214184/gallery_04.webp;/upload/vvm_images/import_images/214184/gallery_05.webp;/upload/vvm_images/import_images/214184/gallery_06.webp;/upload/vvm_images/import_images/214184/gallery_07.webp;/upload/vvm_images/import_images/214184/gallery_08.webp;/upload/vvm_images/import_images/214184/gallery_09.webp;/upload/vvm_images/import_images/214184/gallery_10.webp;/upload/vvm_images/import_images/214184/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -1087,7 +991,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/214185/gallery_01.webp|/upload/vvm_images/import_images/214185/gallery_02.webp|/upload/vvm_images/import_images/214185/gallery_03.webp|/upload/vvm_images/import_images/214185/gallery_04.webp|/upload/vvm_images/import_images/214185/gallery_05.webp|/upload/vvm_images/import_images/214185/gallery_06.webp|/upload/vvm_images/import_images/214185/gallery_07.webp|/upload/vvm_images/import_images/214185/gallery_08.webp|/upload/vvm_images/import_images/214185/gallery_09.webp|/upload/vvm_images/import_images/214185/gallery_10.webp|/upload/vvm_images/import_images/214185/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/214185/gallery_01.webp;/upload/vvm_images/import_images/214185/gallery_02.webp;/upload/vvm_images/import_images/214185/gallery_03.webp;/upload/vvm_images/import_images/214185/gallery_04.webp;/upload/vvm_images/import_images/214185/gallery_05.webp;/upload/vvm_images/import_images/214185/gallery_06.webp;/upload/vvm_images/import_images/214185/gallery_07.webp;/upload/vvm_images/import_images/214185/gallery_08.webp;/upload/vvm_images/import_images/214185/gallery_09.webp;/upload/vvm_images/import_images/214185/gallery_10.webp;/upload/vvm_images/import_images/214185/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -1102,11 +1006,7 @@
           <t>/upload/vvm_images/import_images/209205/preview.webp</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/209205/nan</t>
-        </is>
-      </c>
+      <c r="C40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1121,7 +1021,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205583/gallery_01.webp|/upload/vvm_images/import_images/205583/gallery_02.webp|/upload/vvm_images/import_images/205583/gallery_03.webp|/upload/vvm_images/import_images/205583/gallery_04.webp|/upload/vvm_images/import_images/205583/gallery_05.webp|/upload/vvm_images/import_images/205583/gallery_06.webp|/upload/vvm_images/import_images/205583/gallery_07.webp</t>
+          <t>/upload/vvm_images/import_images/205583/gallery_01.webp;/upload/vvm_images/import_images/205583/gallery_02.webp;/upload/vvm_images/import_images/205583/gallery_03.webp;/upload/vvm_images/import_images/205583/gallery_04.webp;/upload/vvm_images/import_images/205583/gallery_05.webp;/upload/vvm_images/import_images/205583/gallery_06.webp;/upload/vvm_images/import_images/205583/gallery_07.webp</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1038,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205584/gallery_01.webp|/upload/vvm_images/import_images/205584/gallery_02.webp|/upload/vvm_images/import_images/205584/gallery_03.webp|/upload/vvm_images/import_images/205584/gallery_04.webp|/upload/vvm_images/import_images/205584/gallery_05.webp|/upload/vvm_images/import_images/205584/gallery_06.webp|/upload/vvm_images/import_images/205584/gallery_07.webp|/upload/vvm_images/import_images/205584/gallery_08.webp</t>
+          <t>/upload/vvm_images/import_images/205584/gallery_01.webp;/upload/vvm_images/import_images/205584/gallery_02.webp;/upload/vvm_images/import_images/205584/gallery_03.webp;/upload/vvm_images/import_images/205584/gallery_04.webp;/upload/vvm_images/import_images/205584/gallery_05.webp;/upload/vvm_images/import_images/205584/gallery_06.webp;/upload/vvm_images/import_images/205584/gallery_07.webp;/upload/vvm_images/import_images/205584/gallery_08.webp</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1055,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205582/gallery_01.webp|/upload/vvm_images/import_images/205582/gallery_02.webp|/upload/vvm_images/import_images/205582/gallery_03.webp|/upload/vvm_images/import_images/205582/gallery_04.webp|/upload/vvm_images/import_images/205582/gallery_05.webp|/upload/vvm_images/import_images/205582/gallery_06.webp|/upload/vvm_images/import_images/205582/gallery_07.webp|/upload/vvm_images/import_images/205582/gallery_08.webp</t>
+          <t>/upload/vvm_images/import_images/205582/gallery_01.webp;/upload/vvm_images/import_images/205582/gallery_02.webp;/upload/vvm_images/import_images/205582/gallery_03.webp;/upload/vvm_images/import_images/205582/gallery_04.webp;/upload/vvm_images/import_images/205582/gallery_05.webp;/upload/vvm_images/import_images/205582/gallery_06.webp;/upload/vvm_images/import_images/205582/gallery_07.webp;/upload/vvm_images/import_images/205582/gallery_08.webp</t>
         </is>
       </c>
     </row>
@@ -1170,11 +1070,7 @@
           <t>/upload/vvm_images/import_images/186615/preview.webp</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/186615/nan</t>
-        </is>
-      </c>
+      <c r="C44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1187,11 +1083,7 @@
           <t>/upload/vvm_images/import_images/186616/preview.webp</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/186616/nan</t>
-        </is>
-      </c>
+      <c r="C45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1204,11 +1096,7 @@
           <t>/upload/vvm_images/import_images/186613/preview.webp</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/186613/nan</t>
-        </is>
-      </c>
+      <c r="C46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1221,11 +1109,7 @@
           <t>/upload/vvm_images/import_images/186614/preview.webp</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/186614/nan</t>
-        </is>
-      </c>
+      <c r="C47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1238,11 +1122,7 @@
           <t>/upload/vvm_images/import_images/184651/preview.webp</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184651/nan</t>
-        </is>
-      </c>
+      <c r="C48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1255,11 +1135,7 @@
           <t>/upload/vvm_images/import_images/198552/preview.webp</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198552/nan</t>
-        </is>
-      </c>
+      <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1272,11 +1148,7 @@
           <t>/upload/vvm_images/import_images/198544/preview.webp</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198544/nan</t>
-        </is>
-      </c>
+      <c r="C50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1289,11 +1161,7 @@
           <t>/upload/vvm_images/import_images/184658/preview.webp</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184658/nan</t>
-        </is>
-      </c>
+      <c r="C51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1306,11 +1174,7 @@
           <t>/upload/vvm_images/import_images/188220/preview.webp</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/188220/nan</t>
-        </is>
-      </c>
+      <c r="C52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1323,11 +1187,7 @@
           <t>/upload/vvm_images/import_images/198553/preview.webp</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198553/nan</t>
-        </is>
-      </c>
+      <c r="C53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1340,11 +1200,7 @@
           <t>/upload/vvm_images/import_images/184660/preview.webp</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184660/nan</t>
-        </is>
-      </c>
+      <c r="C54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1357,11 +1213,7 @@
           <t>/upload/vvm_images/import_images/184662/preview.webp</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184662/nan</t>
-        </is>
-      </c>
+      <c r="C55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1374,11 +1226,7 @@
           <t>/upload/vvm_images/import_images/184663/preview.webp</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184663/nan</t>
-        </is>
-      </c>
+      <c r="C56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1391,11 +1239,7 @@
           <t>/upload/vvm_images/import_images/198554/preview.webp</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198554/nan</t>
-        </is>
-      </c>
+      <c r="C57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1408,11 +1252,7 @@
           <t>/upload/vvm_images/import_images/184664/preview.webp</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184664/nan</t>
-        </is>
-      </c>
+      <c r="C58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1425,11 +1265,7 @@
           <t>/upload/vvm_images/import_images/184666/preview.webp</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184666/nan</t>
-        </is>
-      </c>
+      <c r="C59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1442,11 +1278,7 @@
           <t>/upload/vvm_images/import_images/184667/preview.webp</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184667/nan</t>
-        </is>
-      </c>
+      <c r="C60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1459,11 +1291,7 @@
           <t>/upload/vvm_images/import_images/198555/preview.webp</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198555/nan</t>
-        </is>
-      </c>
+      <c r="C61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1476,11 +1304,7 @@
           <t>/upload/vvm_images/import_images/188221/preview.webp</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/188221/nan</t>
-        </is>
-      </c>
+      <c r="C62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1493,11 +1317,7 @@
           <t>/upload/vvm_images/import_images/184670/preview.webp</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184670/nan</t>
-        </is>
-      </c>
+      <c r="C63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1510,11 +1330,7 @@
           <t>/upload/vvm_images/import_images/188222/preview.webp</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/188222/nan</t>
-        </is>
-      </c>
+      <c r="C64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1527,11 +1343,7 @@
           <t>/upload/vvm_images/import_images/198556/preview.webp</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198556/nan</t>
-        </is>
-      </c>
+      <c r="C65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1544,11 +1356,7 @@
           <t>/upload/vvm_images/import_images/184672/preview.webp</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/184672/nan</t>
-        </is>
-      </c>
+      <c r="C66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1561,11 +1369,7 @@
           <t>/upload/vvm_images/import_images/198551/preview.webp</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198551/nan</t>
-        </is>
-      </c>
+      <c r="C67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1578,11 +1382,7 @@
           <t>/upload/vvm_images/import_images/205590/preview.webp</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205590/nan</t>
-        </is>
-      </c>
+      <c r="C68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1595,11 +1395,7 @@
           <t>/upload/vvm_images/import_images/188225/preview.webp</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/188225/nan</t>
-        </is>
-      </c>
+      <c r="C69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1612,11 +1408,7 @@
           <t>/upload/vvm_images/import_images/205560/preview.webp</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205560/nan</t>
-        </is>
-      </c>
+      <c r="C70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1631,7 +1423,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205587/gallery_01.webp|/upload/vvm_images/import_images/205587/gallery_02.webp|/upload/vvm_images/import_images/205587/gallery_03.webp|/upload/vvm_images/import_images/205587/gallery_04.webp|/upload/vvm_images/import_images/205587/gallery_05.webp|/upload/vvm_images/import_images/205587/gallery_06.webp</t>
+          <t>/upload/vvm_images/import_images/205587/gallery_01.webp;/upload/vvm_images/import_images/205587/gallery_02.webp;/upload/vvm_images/import_images/205587/gallery_03.webp;/upload/vvm_images/import_images/205587/gallery_04.webp;/upload/vvm_images/import_images/205587/gallery_05.webp;/upload/vvm_images/import_images/205587/gallery_06.webp</t>
         </is>
       </c>
     </row>
@@ -1646,11 +1438,7 @@
           <t>/upload/vvm_images/import_images/205601/preview.webp</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205601/nan</t>
-        </is>
-      </c>
+      <c r="C72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1663,11 +1451,7 @@
           <t>/upload/vvm_images/import_images/191611/preview.webp</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/191611/nan</t>
-        </is>
-      </c>
+      <c r="C73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1680,11 +1464,7 @@
           <t>/upload/vvm_images/import_images/198041/preview.webp</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/198041/nan</t>
-        </is>
-      </c>
+      <c r="C74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1697,11 +1477,7 @@
           <t>/upload/vvm_images/import_images/202413/preview.webp</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/202413/nan</t>
-        </is>
-      </c>
+      <c r="C75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1714,11 +1490,7 @@
           <t>/upload/vvm_images/import_images/204842/preview.webp</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204842/nan</t>
-        </is>
-      </c>
+      <c r="C76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1731,11 +1503,7 @@
           <t>/upload/vvm_images/import_images/205716/preview.webp</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205716/nan</t>
-        </is>
-      </c>
+      <c r="C77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1748,11 +1516,7 @@
           <t>/upload/vvm_images/import_images/205721/preview.webp</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205721/nan</t>
-        </is>
-      </c>
+      <c r="C78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1767,7 +1531,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205726/gallery_01.webp|/upload/vvm_images/import_images/205726/gallery_02.webp|/upload/vvm_images/import_images/205726/gallery_03.webp|/upload/vvm_images/import_images/205726/gallery_04.webp|/upload/vvm_images/import_images/205726/gallery_05.webp|/upload/vvm_images/import_images/205726/gallery_06.webp|/upload/vvm_images/import_images/205726/gallery_07.webp|/upload/vvm_images/import_images/205726/gallery_08.webp|/upload/vvm_images/import_images/205726/gallery_09.webp|/upload/vvm_images/import_images/205726/gallery_10.webp|/upload/vvm_images/import_images/205726/gallery_11.webp|/upload/vvm_images/import_images/205726/gallery_12.webp|/upload/vvm_images/import_images/205726/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/205726/gallery_01.webp;/upload/vvm_images/import_images/205726/gallery_02.webp;/upload/vvm_images/import_images/205726/gallery_03.webp;/upload/vvm_images/import_images/205726/gallery_04.webp;/upload/vvm_images/import_images/205726/gallery_05.webp;/upload/vvm_images/import_images/205726/gallery_06.webp;/upload/vvm_images/import_images/205726/gallery_07.webp;/upload/vvm_images/import_images/205726/gallery_08.webp;/upload/vvm_images/import_images/205726/gallery_09.webp;/upload/vvm_images/import_images/205726/gallery_10.webp;/upload/vvm_images/import_images/205726/gallery_11.webp;/upload/vvm_images/import_images/205726/gallery_12.webp;/upload/vvm_images/import_images/205726/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1548,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205776/gallery_01.webp|/upload/vvm_images/import_images/205776/gallery_02.webp|/upload/vvm_images/import_images/205776/gallery_03.webp|/upload/vvm_images/import_images/205776/gallery_04.webp|/upload/vvm_images/import_images/205776/gallery_05.webp|/upload/vvm_images/import_images/205776/gallery_06.webp|/upload/vvm_images/import_images/205776/gallery_07.webp|/upload/vvm_images/import_images/205776/gallery_08.webp|/upload/vvm_images/import_images/205776/gallery_09.webp|/upload/vvm_images/import_images/205776/gallery_10.webp|/upload/vvm_images/import_images/205776/gallery_11.webp|/upload/vvm_images/import_images/205776/gallery_12.webp</t>
+          <t>/upload/vvm_images/import_images/205776/gallery_01.webp;/upload/vvm_images/import_images/205776/gallery_02.webp;/upload/vvm_images/import_images/205776/gallery_03.webp;/upload/vvm_images/import_images/205776/gallery_04.webp;/upload/vvm_images/import_images/205776/gallery_05.webp;/upload/vvm_images/import_images/205776/gallery_06.webp;/upload/vvm_images/import_images/205776/gallery_07.webp;/upload/vvm_images/import_images/205776/gallery_08.webp;/upload/vvm_images/import_images/205776/gallery_09.webp;/upload/vvm_images/import_images/205776/gallery_10.webp;/upload/vvm_images/import_images/205776/gallery_11.webp;/upload/vvm_images/import_images/205776/gallery_12.webp</t>
         </is>
       </c>
     </row>
@@ -1799,11 +1563,7 @@
           <t>/upload/vvm_images/import_images/211351/preview.webp</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/211351/nan</t>
-        </is>
-      </c>
+      <c r="C81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1816,11 +1576,7 @@
           <t>/upload/vvm_images/import_images/179136/preview.webp</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/179136/nan</t>
-        </is>
-      </c>
+      <c r="C82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1833,11 +1589,7 @@
           <t>/upload/vvm_images/import_images/174459/preview.webp</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/174459/nan</t>
-        </is>
-      </c>
+      <c r="C83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1852,7 +1604,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/198648/gallery_01.webp|/upload/vvm_images/import_images/198648/gallery_02.webp|/upload/vvm_images/import_images/198648/gallery_03.webp|/upload/vvm_images/import_images/198648/gallery_04.webp|/upload/vvm_images/import_images/198648/gallery_05.webp|/upload/vvm_images/import_images/198648/gallery_06.webp|/upload/vvm_images/import_images/198648/gallery_07.webp|/upload/vvm_images/import_images/198648/gallery_08.webp|/upload/vvm_images/import_images/198648/gallery_09.webp|/upload/vvm_images/import_images/198648/gallery_10.webp|/upload/vvm_images/import_images/198648/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/198648/gallery_01.webp;/upload/vvm_images/import_images/198648/gallery_02.webp;/upload/vvm_images/import_images/198648/gallery_03.webp;/upload/vvm_images/import_images/198648/gallery_04.webp;/upload/vvm_images/import_images/198648/gallery_05.webp;/upload/vvm_images/import_images/198648/gallery_06.webp;/upload/vvm_images/import_images/198648/gallery_07.webp;/upload/vvm_images/import_images/198648/gallery_08.webp;/upload/vvm_images/import_images/198648/gallery_09.webp;/upload/vvm_images/import_images/198648/gallery_10.webp;/upload/vvm_images/import_images/198648/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -1867,11 +1619,7 @@
           <t>/upload/vvm_images/import_images/205962/preview.webp</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205962/nan</t>
-        </is>
-      </c>
+      <c r="C85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1884,11 +1632,7 @@
           <t>/upload/vvm_images/import_images/205964/preview.webp</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205964/nan</t>
-        </is>
-      </c>
+      <c r="C86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1903,7 +1647,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/198651/gallery_01.webp|/upload/vvm_images/import_images/198651/gallery_02.webp|/upload/vvm_images/import_images/198651/gallery_03.webp|/upload/vvm_images/import_images/198651/gallery_04.webp|/upload/vvm_images/import_images/198651/gallery_05.webp|/upload/vvm_images/import_images/198651/gallery_06.webp|/upload/vvm_images/import_images/198651/gallery_07.webp|/upload/vvm_images/import_images/198651/gallery_08.webp|/upload/vvm_images/import_images/198651/gallery_09.webp|/upload/vvm_images/import_images/198651/gallery_10.webp|/upload/vvm_images/import_images/198651/gallery_11.webp|/upload/vvm_images/import_images/198651/gallery_12.webp</t>
+          <t>/upload/vvm_images/import_images/198651/gallery_01.webp;/upload/vvm_images/import_images/198651/gallery_02.webp;/upload/vvm_images/import_images/198651/gallery_03.webp;/upload/vvm_images/import_images/198651/gallery_04.webp;/upload/vvm_images/import_images/198651/gallery_05.webp;/upload/vvm_images/import_images/198651/gallery_06.webp;/upload/vvm_images/import_images/198651/gallery_07.webp;/upload/vvm_images/import_images/198651/gallery_08.webp;/upload/vvm_images/import_images/198651/gallery_09.webp;/upload/vvm_images/import_images/198651/gallery_10.webp;/upload/vvm_images/import_images/198651/gallery_11.webp;/upload/vvm_images/import_images/198651/gallery_12.webp</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1664,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205968/gallery_01.webp|/upload/vvm_images/import_images/205968/gallery_02.webp|/upload/vvm_images/import_images/205968/gallery_03.webp|/upload/vvm_images/import_images/205968/gallery_04.webp|/upload/vvm_images/import_images/205968/gallery_05.webp|/upload/vvm_images/import_images/205968/gallery_06.webp|/upload/vvm_images/import_images/205968/gallery_07.webp|/upload/vvm_images/import_images/205968/gallery_08.webp|/upload/vvm_images/import_images/205968/gallery_09.webp|/upload/vvm_images/import_images/205968/gallery_10.webp|/upload/vvm_images/import_images/205968/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/205968/gallery_01.webp;/upload/vvm_images/import_images/205968/gallery_02.webp;/upload/vvm_images/import_images/205968/gallery_03.webp;/upload/vvm_images/import_images/205968/gallery_04.webp;/upload/vvm_images/import_images/205968/gallery_05.webp;/upload/vvm_images/import_images/205968/gallery_06.webp;/upload/vvm_images/import_images/205968/gallery_07.webp;/upload/vvm_images/import_images/205968/gallery_08.webp;/upload/vvm_images/import_images/205968/gallery_09.webp;/upload/vvm_images/import_images/205968/gallery_10.webp;/upload/vvm_images/import_images/205968/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1681,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205969/gallery_01.webp|/upload/vvm_images/import_images/205969/gallery_02.webp|/upload/vvm_images/import_images/205969/gallery_03.webp|/upload/vvm_images/import_images/205969/gallery_04.webp|/upload/vvm_images/import_images/205969/gallery_05.webp|/upload/vvm_images/import_images/205969/gallery_06.webp|/upload/vvm_images/import_images/205969/gallery_07.webp|/upload/vvm_images/import_images/205969/gallery_08.webp|/upload/vvm_images/import_images/205969/gallery_09.webp|/upload/vvm_images/import_images/205969/gallery_10.webp|/upload/vvm_images/import_images/205969/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/205969/gallery_01.webp;/upload/vvm_images/import_images/205969/gallery_02.webp;/upload/vvm_images/import_images/205969/gallery_03.webp;/upload/vvm_images/import_images/205969/gallery_04.webp;/upload/vvm_images/import_images/205969/gallery_05.webp;/upload/vvm_images/import_images/205969/gallery_06.webp;/upload/vvm_images/import_images/205969/gallery_07.webp;/upload/vvm_images/import_images/205969/gallery_08.webp;/upload/vvm_images/import_images/205969/gallery_09.webp;/upload/vvm_images/import_images/205969/gallery_10.webp;/upload/vvm_images/import_images/205969/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -1952,11 +1696,7 @@
           <t>/upload/vvm_images/import_images/201948/preview.webp</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/201948/nan</t>
-        </is>
-      </c>
+      <c r="C90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1969,11 +1709,7 @@
           <t>/upload/vvm_images/import_images/201952/preview.webp</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/201952/nan</t>
-        </is>
-      </c>
+      <c r="C91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1986,11 +1722,7 @@
           <t>/upload/vvm_images/import_images/201956/preview.webp</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/201956/nan</t>
-        </is>
-      </c>
+      <c r="C92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2005,7 +1737,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207362/gallery_01.webp|/upload/vvm_images/import_images/207362/gallery_02.webp|/upload/vvm_images/import_images/207362/gallery_03.webp|/upload/vvm_images/import_images/207362/gallery_04.webp|/upload/vvm_images/import_images/207362/gallery_05.webp|/upload/vvm_images/import_images/207362/gallery_06.webp|/upload/vvm_images/import_images/207362/gallery_07.webp|/upload/vvm_images/import_images/207362/gallery_08.webp|/upload/vvm_images/import_images/207362/gallery_09.webp|/upload/vvm_images/import_images/207362/gallery_10.webp|/upload/vvm_images/import_images/207362/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/207362/gallery_01.webp;/upload/vvm_images/import_images/207362/gallery_02.webp;/upload/vvm_images/import_images/207362/gallery_03.webp;/upload/vvm_images/import_images/207362/gallery_04.webp;/upload/vvm_images/import_images/207362/gallery_05.webp;/upload/vvm_images/import_images/207362/gallery_06.webp;/upload/vvm_images/import_images/207362/gallery_07.webp;/upload/vvm_images/import_images/207362/gallery_08.webp;/upload/vvm_images/import_images/207362/gallery_09.webp;/upload/vvm_images/import_images/207362/gallery_10.webp;/upload/vvm_images/import_images/207362/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -2022,7 +1754,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207363/gallery_01.webp|/upload/vvm_images/import_images/207363/gallery_02.webp|/upload/vvm_images/import_images/207363/gallery_03.webp|/upload/vvm_images/import_images/207363/gallery_04.webp|/upload/vvm_images/import_images/207363/gallery_05.webp|/upload/vvm_images/import_images/207363/gallery_06.webp|/upload/vvm_images/import_images/207363/gallery_07.webp|/upload/vvm_images/import_images/207363/gallery_08.webp|/upload/vvm_images/import_images/207363/gallery_09.webp|/upload/vvm_images/import_images/207363/gallery_10.webp|/upload/vvm_images/import_images/207363/gallery_11.webp|/upload/vvm_images/import_images/207363/gallery_12.webp|/upload/vvm_images/import_images/207363/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207363/gallery_01.webp;/upload/vvm_images/import_images/207363/gallery_02.webp;/upload/vvm_images/import_images/207363/gallery_03.webp;/upload/vvm_images/import_images/207363/gallery_04.webp;/upload/vvm_images/import_images/207363/gallery_05.webp;/upload/vvm_images/import_images/207363/gallery_06.webp;/upload/vvm_images/import_images/207363/gallery_07.webp;/upload/vvm_images/import_images/207363/gallery_08.webp;/upload/vvm_images/import_images/207363/gallery_09.webp;/upload/vvm_images/import_images/207363/gallery_10.webp;/upload/vvm_images/import_images/207363/gallery_11.webp;/upload/vvm_images/import_images/207363/gallery_12.webp;/upload/vvm_images/import_images/207363/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2039,7 +1771,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207364/gallery_01.webp|/upload/vvm_images/import_images/207364/gallery_02.webp|/upload/vvm_images/import_images/207364/gallery_03.webp|/upload/vvm_images/import_images/207364/gallery_04.webp|/upload/vvm_images/import_images/207364/gallery_05.webp|/upload/vvm_images/import_images/207364/gallery_06.webp|/upload/vvm_images/import_images/207364/gallery_07.webp|/upload/vvm_images/import_images/207364/gallery_08.webp|/upload/vvm_images/import_images/207364/gallery_09.webp|/upload/vvm_images/import_images/207364/gallery_10.webp|/upload/vvm_images/import_images/207364/gallery_11.webp|/upload/vvm_images/import_images/207364/gallery_12.webp|/upload/vvm_images/import_images/207364/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207364/gallery_01.webp;/upload/vvm_images/import_images/207364/gallery_02.webp;/upload/vvm_images/import_images/207364/gallery_03.webp;/upload/vvm_images/import_images/207364/gallery_04.webp;/upload/vvm_images/import_images/207364/gallery_05.webp;/upload/vvm_images/import_images/207364/gallery_06.webp;/upload/vvm_images/import_images/207364/gallery_07.webp;/upload/vvm_images/import_images/207364/gallery_08.webp;/upload/vvm_images/import_images/207364/gallery_09.webp;/upload/vvm_images/import_images/207364/gallery_10.webp;/upload/vvm_images/import_images/207364/gallery_11.webp;/upload/vvm_images/import_images/207364/gallery_12.webp;/upload/vvm_images/import_images/207364/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2054,11 +1786,7 @@
           <t>/upload/vvm_images/import_images/199137/preview.webp</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/199137/nan</t>
-        </is>
-      </c>
+      <c r="C96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2071,11 +1799,7 @@
           <t>/upload/vvm_images/import_images/199138/preview.webp</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/199138/nan</t>
-        </is>
-      </c>
+      <c r="C97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2088,11 +1812,7 @@
           <t>/upload/vvm_images/import_images/200368/preview.webp</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/200368/nan</t>
-        </is>
-      </c>
+      <c r="C98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2105,11 +1825,7 @@
           <t>/upload/vvm_images/import_images/200363/preview.webp</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/200363/nan</t>
-        </is>
-      </c>
+      <c r="C99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2122,11 +1838,7 @@
           <t>/upload/vvm_images/import_images/200364/preview.webp</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/200364/nan</t>
-        </is>
-      </c>
+      <c r="C100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2139,11 +1851,7 @@
           <t>/upload/vvm_images/import_images/200366/preview.webp</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/200366/nan</t>
-        </is>
-      </c>
+      <c r="C101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2156,11 +1864,7 @@
           <t>/upload/vvm_images/import_images/200361/preview.webp</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/200361/nan</t>
-        </is>
-      </c>
+      <c r="C102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2173,11 +1877,7 @@
           <t>/upload/vvm_images/import_images/207384/preview.webp</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/207384/nan</t>
-        </is>
-      </c>
+      <c r="C103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2190,11 +1890,7 @@
           <t>/upload/vvm_images/import_images/206486/preview.webp</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/206486/nan</t>
-        </is>
-      </c>
+      <c r="C104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2207,11 +1903,7 @@
           <t>/upload/vvm_images/import_images/206487/preview.webp</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/206487/nan</t>
-        </is>
-      </c>
+      <c r="C105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2224,11 +1916,7 @@
           <t>/upload/vvm_images/import_images/206488/preview.webp</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/206488/nan</t>
-        </is>
-      </c>
+      <c r="C106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2241,11 +1929,7 @@
           <t>/upload/vvm_images/import_images/214916/preview.webp</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/214916/nan</t>
-        </is>
-      </c>
+      <c r="C107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2258,11 +1942,7 @@
           <t>/upload/vvm_images/import_images/214918/preview.webp</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/214918/nan</t>
-        </is>
-      </c>
+      <c r="C108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2275,11 +1955,7 @@
           <t>/upload/vvm_images/import_images/211398/preview.webp</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/211398/nan</t>
-        </is>
-      </c>
+      <c r="C109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2292,11 +1968,7 @@
           <t>/upload/vvm_images/import_images/211399/preview.webp</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/211399/nan</t>
-        </is>
-      </c>
+      <c r="C110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2311,7 +1983,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204005/gallery_01.webp|/upload/vvm_images/import_images/204005/gallery_02.webp|/upload/vvm_images/import_images/204005/gallery_03.webp|/upload/vvm_images/import_images/204005/gallery_04.webp|/upload/vvm_images/import_images/204005/gallery_05.webp|/upload/vvm_images/import_images/204005/gallery_06.webp|/upload/vvm_images/import_images/204005/gallery_07.webp|/upload/vvm_images/import_images/204005/gallery_08.webp|/upload/vvm_images/import_images/204005/gallery_09.webp|/upload/vvm_images/import_images/204005/gallery_10.webp|/upload/vvm_images/import_images/204005/gallery_11.webp|/upload/vvm_images/import_images/204005/gallery_12.webp|/upload/vvm_images/import_images/204005/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/204005/gallery_01.webp;/upload/vvm_images/import_images/204005/gallery_02.webp;/upload/vvm_images/import_images/204005/gallery_03.webp;/upload/vvm_images/import_images/204005/gallery_04.webp;/upload/vvm_images/import_images/204005/gallery_05.webp;/upload/vvm_images/import_images/204005/gallery_06.webp;/upload/vvm_images/import_images/204005/gallery_07.webp;/upload/vvm_images/import_images/204005/gallery_08.webp;/upload/vvm_images/import_images/204005/gallery_09.webp;/upload/vvm_images/import_images/204005/gallery_10.webp;/upload/vvm_images/import_images/204005/gallery_11.webp;/upload/vvm_images/import_images/204005/gallery_12.webp;/upload/vvm_images/import_images/204005/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2000,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210312/gallery_01.webp|/upload/vvm_images/import_images/210312/gallery_02.webp|/upload/vvm_images/import_images/210312/gallery_03.webp|/upload/vvm_images/import_images/210312/gallery_04.webp|/upload/vvm_images/import_images/210312/gallery_05.webp|/upload/vvm_images/import_images/210312/gallery_06.webp|/upload/vvm_images/import_images/210312/gallery_07.webp|/upload/vvm_images/import_images/210312/gallery_08.webp|/upload/vvm_images/import_images/210312/gallery_09.webp|/upload/vvm_images/import_images/210312/gallery_10.webp|/upload/vvm_images/import_images/210312/gallery_11.webp|/upload/vvm_images/import_images/210312/gallery_12.webp|/upload/vvm_images/import_images/210312/gallery_13.webp|/upload/vvm_images/import_images/210312/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/210312/gallery_01.webp;/upload/vvm_images/import_images/210312/gallery_02.webp;/upload/vvm_images/import_images/210312/gallery_03.webp;/upload/vvm_images/import_images/210312/gallery_04.webp;/upload/vvm_images/import_images/210312/gallery_05.webp;/upload/vvm_images/import_images/210312/gallery_06.webp;/upload/vvm_images/import_images/210312/gallery_07.webp;/upload/vvm_images/import_images/210312/gallery_08.webp;/upload/vvm_images/import_images/210312/gallery_09.webp;/upload/vvm_images/import_images/210312/gallery_10.webp;/upload/vvm_images/import_images/210312/gallery_11.webp;/upload/vvm_images/import_images/210312/gallery_12.webp;/upload/vvm_images/import_images/210312/gallery_13.webp;/upload/vvm_images/import_images/210312/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2017,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204882/gallery_01.webp|/upload/vvm_images/import_images/204882/gallery_02.webp|/upload/vvm_images/import_images/204882/gallery_03.webp|/upload/vvm_images/import_images/204882/gallery_04.webp|/upload/vvm_images/import_images/204882/gallery_05.webp|/upload/vvm_images/import_images/204882/gallery_06.webp|/upload/vvm_images/import_images/204882/gallery_07.webp|/upload/vvm_images/import_images/204882/gallery_08.webp|/upload/vvm_images/import_images/204882/gallery_09.webp|/upload/vvm_images/import_images/204882/gallery_10.webp|/upload/vvm_images/import_images/204882/gallery_11.webp|/upload/vvm_images/import_images/204882/gallery_12.webp|/upload/vvm_images/import_images/204882/gallery_13.webp|/upload/vvm_images/import_images/204882/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/204882/gallery_01.webp;/upload/vvm_images/import_images/204882/gallery_02.webp;/upload/vvm_images/import_images/204882/gallery_03.webp;/upload/vvm_images/import_images/204882/gallery_04.webp;/upload/vvm_images/import_images/204882/gallery_05.webp;/upload/vvm_images/import_images/204882/gallery_06.webp;/upload/vvm_images/import_images/204882/gallery_07.webp;/upload/vvm_images/import_images/204882/gallery_08.webp;/upload/vvm_images/import_images/204882/gallery_09.webp;/upload/vvm_images/import_images/204882/gallery_10.webp;/upload/vvm_images/import_images/204882/gallery_11.webp;/upload/vvm_images/import_images/204882/gallery_12.webp;/upload/vvm_images/import_images/204882/gallery_13.webp;/upload/vvm_images/import_images/204882/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2360,11 +2032,7 @@
           <t>/upload/vvm_images/import_images/204263/preview.webp</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204263/nan</t>
-        </is>
-      </c>
+      <c r="C114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2379,7 +2047,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/206078/gallery_01.webp|/upload/vvm_images/import_images/206078/gallery_02.webp|/upload/vvm_images/import_images/206078/gallery_03.webp|/upload/vvm_images/import_images/206078/gallery_04.webp</t>
+          <t>/upload/vvm_images/import_images/206078/gallery_01.webp;/upload/vvm_images/import_images/206078/gallery_02.webp;/upload/vvm_images/import_images/206078/gallery_03.webp;/upload/vvm_images/import_images/206078/gallery_04.webp</t>
         </is>
       </c>
     </row>
@@ -2394,11 +2062,7 @@
           <t>/upload/vvm_images/import_images/206079/preview.webp</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/206079/nan</t>
-        </is>
-      </c>
+      <c r="C116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2411,11 +2075,7 @@
           <t>/upload/vvm_images/import_images/180468/preview.webp</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/180468/nan</t>
-        </is>
-      </c>
+      <c r="C117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2428,11 +2088,7 @@
           <t>/upload/vvm_images/import_images/180471/preview.webp</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/180471/nan</t>
-        </is>
-      </c>
+      <c r="C118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2445,11 +2101,7 @@
           <t>/upload/vvm_images/import_images/199635/preview.webp</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/199635/nan</t>
-        </is>
-      </c>
+      <c r="C119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2462,11 +2114,7 @@
           <t>/upload/vvm_images/import_images/200569/preview.webp</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/200569/nan</t>
-        </is>
-      </c>
+      <c r="C120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2481,7 +2129,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204860/gallery_01.webp|/upload/vvm_images/import_images/204860/gallery_02.webp|/upload/vvm_images/import_images/204860/gallery_03.webp|/upload/vvm_images/import_images/204860/gallery_04.webp|/upload/vvm_images/import_images/204860/gallery_05.webp|/upload/vvm_images/import_images/204860/gallery_06.webp|/upload/vvm_images/import_images/204860/gallery_07.webp|/upload/vvm_images/import_images/204860/gallery_08.webp|/upload/vvm_images/import_images/204860/gallery_09.webp|/upload/vvm_images/import_images/204860/gallery_10.webp</t>
+          <t>/upload/vvm_images/import_images/204860/gallery_01.webp;/upload/vvm_images/import_images/204860/gallery_02.webp;/upload/vvm_images/import_images/204860/gallery_03.webp;/upload/vvm_images/import_images/204860/gallery_04.webp;/upload/vvm_images/import_images/204860/gallery_05.webp;/upload/vvm_images/import_images/204860/gallery_06.webp;/upload/vvm_images/import_images/204860/gallery_07.webp;/upload/vvm_images/import_images/204860/gallery_08.webp;/upload/vvm_images/import_images/204860/gallery_09.webp;/upload/vvm_images/import_images/204860/gallery_10.webp</t>
         </is>
       </c>
     </row>
@@ -2496,11 +2144,7 @@
           <t>/upload/vvm_images/import_images/204861/preview.webp</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204861/nan</t>
-        </is>
-      </c>
+      <c r="C122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2515,7 +2159,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204867/gallery_01.webp|/upload/vvm_images/import_images/204867/gallery_02.webp|/upload/vvm_images/import_images/204867/gallery_03.webp|/upload/vvm_images/import_images/204867/gallery_04.webp|/upload/vvm_images/import_images/204867/gallery_05.webp|/upload/vvm_images/import_images/204867/gallery_06.webp|/upload/vvm_images/import_images/204867/gallery_07.webp|/upload/vvm_images/import_images/204867/gallery_08.webp|/upload/vvm_images/import_images/204867/gallery_09.webp|/upload/vvm_images/import_images/204867/gallery_10.webp|/upload/vvm_images/import_images/204867/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/204867/gallery_01.webp;/upload/vvm_images/import_images/204867/gallery_02.webp;/upload/vvm_images/import_images/204867/gallery_03.webp;/upload/vvm_images/import_images/204867/gallery_04.webp;/upload/vvm_images/import_images/204867/gallery_05.webp;/upload/vvm_images/import_images/204867/gallery_06.webp;/upload/vvm_images/import_images/204867/gallery_07.webp;/upload/vvm_images/import_images/204867/gallery_08.webp;/upload/vvm_images/import_images/204867/gallery_09.webp;/upload/vvm_images/import_images/204867/gallery_10.webp;/upload/vvm_images/import_images/204867/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2176,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210283/gallery_01.webp|/upload/vvm_images/import_images/210283/gallery_02.webp|/upload/vvm_images/import_images/210283/gallery_03.webp|/upload/vvm_images/import_images/210283/gallery_04.webp|/upload/vvm_images/import_images/210283/gallery_05.webp|/upload/vvm_images/import_images/210283/gallery_06.webp|/upload/vvm_images/import_images/210283/gallery_07.webp|/upload/vvm_images/import_images/210283/gallery_08.webp|/upload/vvm_images/import_images/210283/gallery_09.webp|/upload/vvm_images/import_images/210283/gallery_10.webp|/upload/vvm_images/import_images/210283/gallery_11.webp|/upload/vvm_images/import_images/210283/gallery_12.webp|/upload/vvm_images/import_images/210283/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/210283/gallery_01.webp;/upload/vvm_images/import_images/210283/gallery_02.webp;/upload/vvm_images/import_images/210283/gallery_03.webp;/upload/vvm_images/import_images/210283/gallery_04.webp;/upload/vvm_images/import_images/210283/gallery_05.webp;/upload/vvm_images/import_images/210283/gallery_06.webp;/upload/vvm_images/import_images/210283/gallery_07.webp;/upload/vvm_images/import_images/210283/gallery_08.webp;/upload/vvm_images/import_images/210283/gallery_09.webp;/upload/vvm_images/import_images/210283/gallery_10.webp;/upload/vvm_images/import_images/210283/gallery_11.webp;/upload/vvm_images/import_images/210283/gallery_12.webp;/upload/vvm_images/import_images/210283/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2227,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205751/gallery_01.webp|/upload/vvm_images/import_images/205751/gallery_02.webp|/upload/vvm_images/import_images/205751/gallery_03.webp|/upload/vvm_images/import_images/205751/gallery_04.webp|/upload/vvm_images/import_images/205751/gallery_05.webp|/upload/vvm_images/import_images/205751/gallery_06.webp|/upload/vvm_images/import_images/205751/gallery_07.webp|/upload/vvm_images/import_images/205751/gallery_08.webp|/upload/vvm_images/import_images/205751/gallery_09.webp|/upload/vvm_images/import_images/205751/gallery_10.webp|/upload/vvm_images/import_images/205751/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/205751/gallery_01.webp;/upload/vvm_images/import_images/205751/gallery_02.webp;/upload/vvm_images/import_images/205751/gallery_03.webp;/upload/vvm_images/import_images/205751/gallery_04.webp;/upload/vvm_images/import_images/205751/gallery_05.webp;/upload/vvm_images/import_images/205751/gallery_06.webp;/upload/vvm_images/import_images/205751/gallery_07.webp;/upload/vvm_images/import_images/205751/gallery_08.webp;/upload/vvm_images/import_images/205751/gallery_09.webp;/upload/vvm_images/import_images/205751/gallery_10.webp;/upload/vvm_images/import_images/205751/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2244,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204508/gallery_01.webp|/upload/vvm_images/import_images/204508/gallery_02.webp|/upload/vvm_images/import_images/204508/gallery_03.webp|/upload/vvm_images/import_images/204508/gallery_04.webp|/upload/vvm_images/import_images/204508/gallery_05.webp|/upload/vvm_images/import_images/204508/gallery_06.webp|/upload/vvm_images/import_images/204508/gallery_07.webp|/upload/vvm_images/import_images/204508/gallery_08.webp|/upload/vvm_images/import_images/204508/gallery_09.webp|/upload/vvm_images/import_images/204508/gallery_10.webp|/upload/vvm_images/import_images/204508/gallery_11.webp|/upload/vvm_images/import_images/204508/gallery_12.webp|/upload/vvm_images/import_images/204508/gallery_13.webp|/upload/vvm_images/import_images/204508/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/204508/gallery_01.webp;/upload/vvm_images/import_images/204508/gallery_02.webp;/upload/vvm_images/import_images/204508/gallery_03.webp;/upload/vvm_images/import_images/204508/gallery_04.webp;/upload/vvm_images/import_images/204508/gallery_05.webp;/upload/vvm_images/import_images/204508/gallery_06.webp;/upload/vvm_images/import_images/204508/gallery_07.webp;/upload/vvm_images/import_images/204508/gallery_08.webp;/upload/vvm_images/import_images/204508/gallery_09.webp;/upload/vvm_images/import_images/204508/gallery_10.webp;/upload/vvm_images/import_images/204508/gallery_11.webp;/upload/vvm_images/import_images/204508/gallery_12.webp;/upload/vvm_images/import_images/204508/gallery_13.webp;/upload/vvm_images/import_images/204508/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2261,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205359/gallery_01.webp|/upload/vvm_images/import_images/205359/gallery_02.webp|/upload/vvm_images/import_images/205359/gallery_03.webp|/upload/vvm_images/import_images/205359/gallery_04.webp|/upload/vvm_images/import_images/205359/gallery_05.webp|/upload/vvm_images/import_images/205359/gallery_06.webp|/upload/vvm_images/import_images/205359/gallery_07.webp|/upload/vvm_images/import_images/205359/gallery_08.webp|/upload/vvm_images/import_images/205359/gallery_09.webp|/upload/vvm_images/import_images/205359/gallery_10.webp|/upload/vvm_images/import_images/205359/gallery_11.webp|/upload/vvm_images/import_images/205359/gallery_12.webp|/upload/vvm_images/import_images/205359/gallery_13.webp|/upload/vvm_images/import_images/205359/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/205359/gallery_01.webp;/upload/vvm_images/import_images/205359/gallery_02.webp;/upload/vvm_images/import_images/205359/gallery_03.webp;/upload/vvm_images/import_images/205359/gallery_04.webp;/upload/vvm_images/import_images/205359/gallery_05.webp;/upload/vvm_images/import_images/205359/gallery_06.webp;/upload/vvm_images/import_images/205359/gallery_07.webp;/upload/vvm_images/import_images/205359/gallery_08.webp;/upload/vvm_images/import_images/205359/gallery_09.webp;/upload/vvm_images/import_images/205359/gallery_10.webp;/upload/vvm_images/import_images/205359/gallery_11.webp;/upload/vvm_images/import_images/205359/gallery_12.webp;/upload/vvm_images/import_images/205359/gallery_13.webp;/upload/vvm_images/import_images/205359/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2278,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205361/gallery_01.webp|/upload/vvm_images/import_images/205361/gallery_02.webp|/upload/vvm_images/import_images/205361/gallery_03.webp|/upload/vvm_images/import_images/205361/gallery_04.webp|/upload/vvm_images/import_images/205361/gallery_05.webp|/upload/vvm_images/import_images/205361/gallery_06.webp|/upload/vvm_images/import_images/205361/gallery_07.webp|/upload/vvm_images/import_images/205361/gallery_08.webp|/upload/vvm_images/import_images/205361/gallery_09.webp|/upload/vvm_images/import_images/205361/gallery_10.webp|/upload/vvm_images/import_images/205361/gallery_11.webp|/upload/vvm_images/import_images/205361/gallery_12.webp|/upload/vvm_images/import_images/205361/gallery_13.webp|/upload/vvm_images/import_images/205361/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/205361/gallery_01.webp;/upload/vvm_images/import_images/205361/gallery_02.webp;/upload/vvm_images/import_images/205361/gallery_03.webp;/upload/vvm_images/import_images/205361/gallery_04.webp;/upload/vvm_images/import_images/205361/gallery_05.webp;/upload/vvm_images/import_images/205361/gallery_06.webp;/upload/vvm_images/import_images/205361/gallery_07.webp;/upload/vvm_images/import_images/205361/gallery_08.webp;/upload/vvm_images/import_images/205361/gallery_09.webp;/upload/vvm_images/import_images/205361/gallery_10.webp;/upload/vvm_images/import_images/205361/gallery_11.webp;/upload/vvm_images/import_images/205361/gallery_12.webp;/upload/vvm_images/import_images/205361/gallery_13.webp;/upload/vvm_images/import_images/205361/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2295,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/191146/gallery_01.webp|/upload/vvm_images/import_images/191146/gallery_02.webp|/upload/vvm_images/import_images/191146/gallery_03.webp|/upload/vvm_images/import_images/191146/gallery_04.webp|/upload/vvm_images/import_images/191146/gallery_05.webp|/upload/vvm_images/import_images/191146/gallery_06.webp|/upload/vvm_images/import_images/191146/gallery_07.webp|/upload/vvm_images/import_images/191146/gallery_08.webp|/upload/vvm_images/import_images/191146/gallery_09.webp|/upload/vvm_images/import_images/191146/gallery_10.webp|/upload/vvm_images/import_images/191146/gallery_11.webp|/upload/vvm_images/import_images/191146/gallery_12.webp|/upload/vvm_images/import_images/191146/gallery_13.webp|/upload/vvm_images/import_images/191146/gallery_14.webp|/upload/vvm_images/import_images/191146/gallery_15.webp</t>
+          <t>/upload/vvm_images/import_images/191146/gallery_01.webp;/upload/vvm_images/import_images/191146/gallery_02.webp;/upload/vvm_images/import_images/191146/gallery_03.webp;/upload/vvm_images/import_images/191146/gallery_04.webp;/upload/vvm_images/import_images/191146/gallery_05.webp;/upload/vvm_images/import_images/191146/gallery_06.webp;/upload/vvm_images/import_images/191146/gallery_07.webp;/upload/vvm_images/import_images/191146/gallery_08.webp;/upload/vvm_images/import_images/191146/gallery_09.webp;/upload/vvm_images/import_images/191146/gallery_10.webp;/upload/vvm_images/import_images/191146/gallery_11.webp;/upload/vvm_images/import_images/191146/gallery_12.webp;/upload/vvm_images/import_images/191146/gallery_13.webp;/upload/vvm_images/import_images/191146/gallery_14.webp;/upload/vvm_images/import_images/191146/gallery_15.webp</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2312,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207403/gallery_01.webp|/upload/vvm_images/import_images/207403/gallery_02.webp|/upload/vvm_images/import_images/207403/gallery_03.webp|/upload/vvm_images/import_images/207403/gallery_04.webp|/upload/vvm_images/import_images/207403/gallery_05.webp|/upload/vvm_images/import_images/207403/gallery_06.webp|/upload/vvm_images/import_images/207403/gallery_07.webp|/upload/vvm_images/import_images/207403/gallery_08.webp|/upload/vvm_images/import_images/207403/gallery_09.webp|/upload/vvm_images/import_images/207403/gallery_10.webp|/upload/vvm_images/import_images/207403/gallery_11.webp|/upload/vvm_images/import_images/207403/gallery_12.webp|/upload/vvm_images/import_images/207403/gallery_13.webp|/upload/vvm_images/import_images/207403/gallery_14.webp|/upload/vvm_images/import_images/207403/gallery_15.webp</t>
+          <t>/upload/vvm_images/import_images/207403/gallery_01.webp;/upload/vvm_images/import_images/207403/gallery_02.webp;/upload/vvm_images/import_images/207403/gallery_03.webp;/upload/vvm_images/import_images/207403/gallery_04.webp;/upload/vvm_images/import_images/207403/gallery_05.webp;/upload/vvm_images/import_images/207403/gallery_06.webp;/upload/vvm_images/import_images/207403/gallery_07.webp;/upload/vvm_images/import_images/207403/gallery_08.webp;/upload/vvm_images/import_images/207403/gallery_09.webp;/upload/vvm_images/import_images/207403/gallery_10.webp;/upload/vvm_images/import_images/207403/gallery_11.webp;/upload/vvm_images/import_images/207403/gallery_12.webp;/upload/vvm_images/import_images/207403/gallery_13.webp;/upload/vvm_images/import_images/207403/gallery_14.webp;/upload/vvm_images/import_images/207403/gallery_15.webp</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2329,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210334/gallery_01.webp|/upload/vvm_images/import_images/210334/gallery_02.webp|/upload/vvm_images/import_images/210334/gallery_03.webp|/upload/vvm_images/import_images/210334/gallery_04.webp|/upload/vvm_images/import_images/210334/gallery_05.webp|/upload/vvm_images/import_images/210334/gallery_06.webp|/upload/vvm_images/import_images/210334/gallery_07.webp|/upload/vvm_images/import_images/210334/gallery_08.webp|/upload/vvm_images/import_images/210334/gallery_09.webp|/upload/vvm_images/import_images/210334/gallery_10.webp|/upload/vvm_images/import_images/210334/gallery_11.webp|/upload/vvm_images/import_images/210334/gallery_12.webp|/upload/vvm_images/import_images/210334/gallery_13.webp|/upload/vvm_images/import_images/210334/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/210334/gallery_01.webp;/upload/vvm_images/import_images/210334/gallery_02.webp;/upload/vvm_images/import_images/210334/gallery_03.webp;/upload/vvm_images/import_images/210334/gallery_04.webp;/upload/vvm_images/import_images/210334/gallery_05.webp;/upload/vvm_images/import_images/210334/gallery_06.webp;/upload/vvm_images/import_images/210334/gallery_07.webp;/upload/vvm_images/import_images/210334/gallery_08.webp;/upload/vvm_images/import_images/210334/gallery_09.webp;/upload/vvm_images/import_images/210334/gallery_10.webp;/upload/vvm_images/import_images/210334/gallery_11.webp;/upload/vvm_images/import_images/210334/gallery_12.webp;/upload/vvm_images/import_images/210334/gallery_13.webp;/upload/vvm_images/import_images/210334/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2346,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210335/gallery_01.webp|/upload/vvm_images/import_images/210335/gallery_02.webp|/upload/vvm_images/import_images/210335/gallery_03.webp|/upload/vvm_images/import_images/210335/gallery_04.webp|/upload/vvm_images/import_images/210335/gallery_05.webp|/upload/vvm_images/import_images/210335/gallery_06.webp|/upload/vvm_images/import_images/210335/gallery_07.webp|/upload/vvm_images/import_images/210335/gallery_08.webp|/upload/vvm_images/import_images/210335/gallery_09.webp|/upload/vvm_images/import_images/210335/gallery_10.webp|/upload/vvm_images/import_images/210335/gallery_11.webp|/upload/vvm_images/import_images/210335/gallery_12.webp|/upload/vvm_images/import_images/210335/gallery_13.webp|/upload/vvm_images/import_images/210335/gallery_14.webp|/upload/vvm_images/import_images/210335/gallery_15.webp|/upload/vvm_images/import_images/210335/gallery_16.webp</t>
+          <t>/upload/vvm_images/import_images/210335/gallery_01.webp;/upload/vvm_images/import_images/210335/gallery_02.webp;/upload/vvm_images/import_images/210335/gallery_03.webp;/upload/vvm_images/import_images/210335/gallery_04.webp;/upload/vvm_images/import_images/210335/gallery_05.webp;/upload/vvm_images/import_images/210335/gallery_06.webp;/upload/vvm_images/import_images/210335/gallery_07.webp;/upload/vvm_images/import_images/210335/gallery_08.webp;/upload/vvm_images/import_images/210335/gallery_09.webp;/upload/vvm_images/import_images/210335/gallery_10.webp;/upload/vvm_images/import_images/210335/gallery_11.webp;/upload/vvm_images/import_images/210335/gallery_12.webp;/upload/vvm_images/import_images/210335/gallery_13.webp;/upload/vvm_images/import_images/210335/gallery_14.webp;/upload/vvm_images/import_images/210335/gallery_15.webp;/upload/vvm_images/import_images/210335/gallery_16.webp</t>
         </is>
       </c>
     </row>
@@ -2717,11 +2361,7 @@
           <t>/upload/vvm_images/import_images/210337/preview.webp</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210337/nan</t>
-        </is>
-      </c>
+      <c r="C135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2736,7 +2376,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207354/gallery_01.webp|/upload/vvm_images/import_images/207354/gallery_02.webp|/upload/vvm_images/import_images/207354/gallery_03.webp|/upload/vvm_images/import_images/207354/gallery_04.webp|/upload/vvm_images/import_images/207354/gallery_05.webp|/upload/vvm_images/import_images/207354/gallery_06.webp|/upload/vvm_images/import_images/207354/gallery_07.webp|/upload/vvm_images/import_images/207354/gallery_08.webp|/upload/vvm_images/import_images/207354/gallery_09.webp|/upload/vvm_images/import_images/207354/gallery_10.webp|/upload/vvm_images/import_images/207354/gallery_11.webp|/upload/vvm_images/import_images/207354/gallery_12.webp|/upload/vvm_images/import_images/207354/gallery_13.webp|/upload/vvm_images/import_images/207354/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/207354/gallery_01.webp;/upload/vvm_images/import_images/207354/gallery_02.webp;/upload/vvm_images/import_images/207354/gallery_03.webp;/upload/vvm_images/import_images/207354/gallery_04.webp;/upload/vvm_images/import_images/207354/gallery_05.webp;/upload/vvm_images/import_images/207354/gallery_06.webp;/upload/vvm_images/import_images/207354/gallery_07.webp;/upload/vvm_images/import_images/207354/gallery_08.webp;/upload/vvm_images/import_images/207354/gallery_09.webp;/upload/vvm_images/import_images/207354/gallery_10.webp;/upload/vvm_images/import_images/207354/gallery_11.webp;/upload/vvm_images/import_images/207354/gallery_12.webp;/upload/vvm_images/import_images/207354/gallery_13.webp;/upload/vvm_images/import_images/207354/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2393,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207355/gallery_01.webp|/upload/vvm_images/import_images/207355/gallery_02.webp|/upload/vvm_images/import_images/207355/gallery_03.webp|/upload/vvm_images/import_images/207355/gallery_04.webp|/upload/vvm_images/import_images/207355/gallery_05.webp|/upload/vvm_images/import_images/207355/gallery_06.webp|/upload/vvm_images/import_images/207355/gallery_07.webp|/upload/vvm_images/import_images/207355/gallery_08.webp|/upload/vvm_images/import_images/207355/gallery_09.webp|/upload/vvm_images/import_images/207355/gallery_10.webp|/upload/vvm_images/import_images/207355/gallery_11.webp|/upload/vvm_images/import_images/207355/gallery_12.webp|/upload/vvm_images/import_images/207355/gallery_13.webp|/upload/vvm_images/import_images/207355/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/207355/gallery_01.webp;/upload/vvm_images/import_images/207355/gallery_02.webp;/upload/vvm_images/import_images/207355/gallery_03.webp;/upload/vvm_images/import_images/207355/gallery_04.webp;/upload/vvm_images/import_images/207355/gallery_05.webp;/upload/vvm_images/import_images/207355/gallery_06.webp;/upload/vvm_images/import_images/207355/gallery_07.webp;/upload/vvm_images/import_images/207355/gallery_08.webp;/upload/vvm_images/import_images/207355/gallery_09.webp;/upload/vvm_images/import_images/207355/gallery_10.webp;/upload/vvm_images/import_images/207355/gallery_11.webp;/upload/vvm_images/import_images/207355/gallery_12.webp;/upload/vvm_images/import_images/207355/gallery_13.webp;/upload/vvm_images/import_images/207355/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -2768,11 +2408,7 @@
           <t>/upload/vvm_images/import_images/211400/preview.webp</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/211400/nan</t>
-        </is>
-      </c>
+      <c r="C138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2787,7 +2423,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207397/gallery_01.webp|/upload/vvm_images/import_images/207397/gallery_02.webp|/upload/vvm_images/import_images/207397/gallery_03.webp|/upload/vvm_images/import_images/207397/gallery_04.webp|/upload/vvm_images/import_images/207397/gallery_05.webp|/upload/vvm_images/import_images/207397/gallery_06.webp|/upload/vvm_images/import_images/207397/gallery_07.webp|/upload/vvm_images/import_images/207397/gallery_08.webp|/upload/vvm_images/import_images/207397/gallery_09.webp|/upload/vvm_images/import_images/207397/gallery_10.webp|/upload/vvm_images/import_images/207397/gallery_11.webp|/upload/vvm_images/import_images/207397/gallery_12.webp|/upload/vvm_images/import_images/207397/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207397/gallery_01.webp;/upload/vvm_images/import_images/207397/gallery_02.webp;/upload/vvm_images/import_images/207397/gallery_03.webp;/upload/vvm_images/import_images/207397/gallery_04.webp;/upload/vvm_images/import_images/207397/gallery_05.webp;/upload/vvm_images/import_images/207397/gallery_06.webp;/upload/vvm_images/import_images/207397/gallery_07.webp;/upload/vvm_images/import_images/207397/gallery_08.webp;/upload/vvm_images/import_images/207397/gallery_09.webp;/upload/vvm_images/import_images/207397/gallery_10.webp;/upload/vvm_images/import_images/207397/gallery_11.webp;/upload/vvm_images/import_images/207397/gallery_12.webp;/upload/vvm_images/import_images/207397/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2440,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207398/gallery_01.webp|/upload/vvm_images/import_images/207398/gallery_02.webp|/upload/vvm_images/import_images/207398/gallery_03.webp|/upload/vvm_images/import_images/207398/gallery_04.webp|/upload/vvm_images/import_images/207398/gallery_05.webp|/upload/vvm_images/import_images/207398/gallery_06.webp|/upload/vvm_images/import_images/207398/gallery_07.webp|/upload/vvm_images/import_images/207398/gallery_08.webp|/upload/vvm_images/import_images/207398/gallery_09.webp|/upload/vvm_images/import_images/207398/gallery_10.webp|/upload/vvm_images/import_images/207398/gallery_11.webp|/upload/vvm_images/import_images/207398/gallery_12.webp|/upload/vvm_images/import_images/207398/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207398/gallery_01.webp;/upload/vvm_images/import_images/207398/gallery_02.webp;/upload/vvm_images/import_images/207398/gallery_03.webp;/upload/vvm_images/import_images/207398/gallery_04.webp;/upload/vvm_images/import_images/207398/gallery_05.webp;/upload/vvm_images/import_images/207398/gallery_06.webp;/upload/vvm_images/import_images/207398/gallery_07.webp;/upload/vvm_images/import_images/207398/gallery_08.webp;/upload/vvm_images/import_images/207398/gallery_09.webp;/upload/vvm_images/import_images/207398/gallery_10.webp;/upload/vvm_images/import_images/207398/gallery_11.webp;/upload/vvm_images/import_images/207398/gallery_12.webp;/upload/vvm_images/import_images/207398/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2457,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207399/gallery_01.webp|/upload/vvm_images/import_images/207399/gallery_02.webp|/upload/vvm_images/import_images/207399/gallery_03.webp|/upload/vvm_images/import_images/207399/gallery_04.webp|/upload/vvm_images/import_images/207399/gallery_05.webp|/upload/vvm_images/import_images/207399/gallery_06.webp|/upload/vvm_images/import_images/207399/gallery_07.webp|/upload/vvm_images/import_images/207399/gallery_08.webp|/upload/vvm_images/import_images/207399/gallery_09.webp|/upload/vvm_images/import_images/207399/gallery_10.webp|/upload/vvm_images/import_images/207399/gallery_11.webp|/upload/vvm_images/import_images/207399/gallery_12.webp|/upload/vvm_images/import_images/207399/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207399/gallery_01.webp;/upload/vvm_images/import_images/207399/gallery_02.webp;/upload/vvm_images/import_images/207399/gallery_03.webp;/upload/vvm_images/import_images/207399/gallery_04.webp;/upload/vvm_images/import_images/207399/gallery_05.webp;/upload/vvm_images/import_images/207399/gallery_06.webp;/upload/vvm_images/import_images/207399/gallery_07.webp;/upload/vvm_images/import_images/207399/gallery_08.webp;/upload/vvm_images/import_images/207399/gallery_09.webp;/upload/vvm_images/import_images/207399/gallery_10.webp;/upload/vvm_images/import_images/207399/gallery_11.webp;/upload/vvm_images/import_images/207399/gallery_12.webp;/upload/vvm_images/import_images/207399/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2474,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207400/gallery_01.webp|/upload/vvm_images/import_images/207400/gallery_02.webp|/upload/vvm_images/import_images/207400/gallery_03.webp|/upload/vvm_images/import_images/207400/gallery_04.webp|/upload/vvm_images/import_images/207400/gallery_05.webp|/upload/vvm_images/import_images/207400/gallery_06.webp|/upload/vvm_images/import_images/207400/gallery_07.webp|/upload/vvm_images/import_images/207400/gallery_08.webp|/upload/vvm_images/import_images/207400/gallery_09.webp|/upload/vvm_images/import_images/207400/gallery_10.webp|/upload/vvm_images/import_images/207400/gallery_11.webp|/upload/vvm_images/import_images/207400/gallery_12.webp|/upload/vvm_images/import_images/207400/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207400/gallery_01.webp;/upload/vvm_images/import_images/207400/gallery_02.webp;/upload/vvm_images/import_images/207400/gallery_03.webp;/upload/vvm_images/import_images/207400/gallery_04.webp;/upload/vvm_images/import_images/207400/gallery_05.webp;/upload/vvm_images/import_images/207400/gallery_06.webp;/upload/vvm_images/import_images/207400/gallery_07.webp;/upload/vvm_images/import_images/207400/gallery_08.webp;/upload/vvm_images/import_images/207400/gallery_09.webp;/upload/vvm_images/import_images/207400/gallery_10.webp;/upload/vvm_images/import_images/207400/gallery_11.webp;/upload/vvm_images/import_images/207400/gallery_12.webp;/upload/vvm_images/import_images/207400/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2491,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207401/gallery_01.webp|/upload/vvm_images/import_images/207401/gallery_02.webp|/upload/vvm_images/import_images/207401/gallery_03.webp|/upload/vvm_images/import_images/207401/gallery_04.webp|/upload/vvm_images/import_images/207401/gallery_05.webp|/upload/vvm_images/import_images/207401/gallery_06.webp|/upload/vvm_images/import_images/207401/gallery_07.webp|/upload/vvm_images/import_images/207401/gallery_08.webp|/upload/vvm_images/import_images/207401/gallery_09.webp|/upload/vvm_images/import_images/207401/gallery_10.webp|/upload/vvm_images/import_images/207401/gallery_11.webp|/upload/vvm_images/import_images/207401/gallery_12.webp|/upload/vvm_images/import_images/207401/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207401/gallery_01.webp;/upload/vvm_images/import_images/207401/gallery_02.webp;/upload/vvm_images/import_images/207401/gallery_03.webp;/upload/vvm_images/import_images/207401/gallery_04.webp;/upload/vvm_images/import_images/207401/gallery_05.webp;/upload/vvm_images/import_images/207401/gallery_06.webp;/upload/vvm_images/import_images/207401/gallery_07.webp;/upload/vvm_images/import_images/207401/gallery_08.webp;/upload/vvm_images/import_images/207401/gallery_09.webp;/upload/vvm_images/import_images/207401/gallery_10.webp;/upload/vvm_images/import_images/207401/gallery_11.webp;/upload/vvm_images/import_images/207401/gallery_12.webp;/upload/vvm_images/import_images/207401/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2508,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207402/gallery_01.webp|/upload/vvm_images/import_images/207402/gallery_02.webp|/upload/vvm_images/import_images/207402/gallery_03.webp|/upload/vvm_images/import_images/207402/gallery_04.webp|/upload/vvm_images/import_images/207402/gallery_05.webp|/upload/vvm_images/import_images/207402/gallery_06.webp|/upload/vvm_images/import_images/207402/gallery_07.webp|/upload/vvm_images/import_images/207402/gallery_08.webp|/upload/vvm_images/import_images/207402/gallery_09.webp|/upload/vvm_images/import_images/207402/gallery_10.webp|/upload/vvm_images/import_images/207402/gallery_11.webp|/upload/vvm_images/import_images/207402/gallery_12.webp|/upload/vvm_images/import_images/207402/gallery_13.webp|/upload/vvm_images/import_images/207402/gallery_14.webp|/upload/vvm_images/import_images/207402/gallery_15.webp</t>
+          <t>/upload/vvm_images/import_images/207402/gallery_01.webp;/upload/vvm_images/import_images/207402/gallery_02.webp;/upload/vvm_images/import_images/207402/gallery_03.webp;/upload/vvm_images/import_images/207402/gallery_04.webp;/upload/vvm_images/import_images/207402/gallery_05.webp;/upload/vvm_images/import_images/207402/gallery_06.webp;/upload/vvm_images/import_images/207402/gallery_07.webp;/upload/vvm_images/import_images/207402/gallery_08.webp;/upload/vvm_images/import_images/207402/gallery_09.webp;/upload/vvm_images/import_images/207402/gallery_10.webp;/upload/vvm_images/import_images/207402/gallery_11.webp;/upload/vvm_images/import_images/207402/gallery_12.webp;/upload/vvm_images/import_images/207402/gallery_13.webp;/upload/vvm_images/import_images/207402/gallery_14.webp;/upload/vvm_images/import_images/207402/gallery_15.webp</t>
         </is>
       </c>
     </row>
@@ -2887,11 +2523,7 @@
           <t>/upload/vvm_images/import_images/202236/preview.webp</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/202236/nan</t>
-        </is>
-      </c>
+      <c r="C145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2906,7 +2538,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/206080/gallery_01.webp|/upload/vvm_images/import_images/206080/gallery_02.webp|/upload/vvm_images/import_images/206080/gallery_03.webp|/upload/vvm_images/import_images/206080/gallery_04.webp|/upload/vvm_images/import_images/206080/gallery_05.webp|/upload/vvm_images/import_images/206080/gallery_06.webp|/upload/vvm_images/import_images/206080/gallery_07.webp|/upload/vvm_images/import_images/206080/gallery_08.webp</t>
+          <t>/upload/vvm_images/import_images/206080/gallery_01.webp;/upload/vvm_images/import_images/206080/gallery_02.webp;/upload/vvm_images/import_images/206080/gallery_03.webp;/upload/vvm_images/import_images/206080/gallery_04.webp;/upload/vvm_images/import_images/206080/gallery_05.webp;/upload/vvm_images/import_images/206080/gallery_06.webp;/upload/vvm_images/import_images/206080/gallery_07.webp;/upload/vvm_images/import_images/206080/gallery_08.webp</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2555,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/206081/gallery_01.webp|/upload/vvm_images/import_images/206081/gallery_02.webp|/upload/vvm_images/import_images/206081/gallery_03.webp|/upload/vvm_images/import_images/206081/gallery_04.webp|/upload/vvm_images/import_images/206081/gallery_05.webp|/upload/vvm_images/import_images/206081/gallery_06.webp|/upload/vvm_images/import_images/206081/gallery_07.webp</t>
+          <t>/upload/vvm_images/import_images/206081/gallery_01.webp;/upload/vvm_images/import_images/206081/gallery_02.webp;/upload/vvm_images/import_images/206081/gallery_03.webp;/upload/vvm_images/import_images/206081/gallery_04.webp;/upload/vvm_images/import_images/206081/gallery_05.webp;/upload/vvm_images/import_images/206081/gallery_06.webp;/upload/vvm_images/import_images/206081/gallery_07.webp</t>
         </is>
       </c>
     </row>
@@ -2938,11 +2570,7 @@
           <t>/upload/vvm_images/import_images/207369/preview.webp</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/207369/nan</t>
-        </is>
-      </c>
+      <c r="C148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2955,11 +2583,7 @@
           <t>/upload/vvm_images/import_images/207370/preview.webp</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/207370/nan</t>
-        </is>
-      </c>
+      <c r="C149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2974,7 +2598,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/185682/gallery_01.webp|/upload/vvm_images/import_images/185682/gallery_02.webp|/upload/vvm_images/import_images/185682/gallery_03.webp|/upload/vvm_images/import_images/185682/gallery_04.webp|/upload/vvm_images/import_images/185682/gallery_05.webp|/upload/vvm_images/import_images/185682/gallery_06.webp|/upload/vvm_images/import_images/185682/gallery_07.webp|/upload/vvm_images/import_images/185682/gallery_08.webp|/upload/vvm_images/import_images/185682/gallery_09.webp|/upload/vvm_images/import_images/185682/gallery_10.webp|/upload/vvm_images/import_images/185682/gallery_11.webp|/upload/vvm_images/import_images/185682/gallery_12.webp|/upload/vvm_images/import_images/185682/gallery_13.webp|/upload/vvm_images/import_images/185682/gallery_14.webp|/upload/vvm_images/import_images/185682/gallery_15.webp</t>
+          <t>/upload/vvm_images/import_images/185682/gallery_01.webp;/upload/vvm_images/import_images/185682/gallery_02.webp;/upload/vvm_images/import_images/185682/gallery_03.webp;/upload/vvm_images/import_images/185682/gallery_04.webp;/upload/vvm_images/import_images/185682/gallery_05.webp;/upload/vvm_images/import_images/185682/gallery_06.webp;/upload/vvm_images/import_images/185682/gallery_07.webp;/upload/vvm_images/import_images/185682/gallery_08.webp;/upload/vvm_images/import_images/185682/gallery_09.webp;/upload/vvm_images/import_images/185682/gallery_10.webp;/upload/vvm_images/import_images/185682/gallery_11.webp;/upload/vvm_images/import_images/185682/gallery_12.webp;/upload/vvm_images/import_images/185682/gallery_13.webp;/upload/vvm_images/import_images/185682/gallery_14.webp;/upload/vvm_images/import_images/185682/gallery_15.webp</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2615,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/214945/gallery_01.webp|/upload/vvm_images/import_images/214945/gallery_02.webp|/upload/vvm_images/import_images/214945/gallery_03.webp|/upload/vvm_images/import_images/214945/gallery_04.webp|/upload/vvm_images/import_images/214945/gallery_05.webp|/upload/vvm_images/import_images/214945/gallery_06.webp|/upload/vvm_images/import_images/214945/gallery_07.webp|/upload/vvm_images/import_images/214945/gallery_08.webp|/upload/vvm_images/import_images/214945/gallery_09.webp</t>
+          <t>/upload/vvm_images/import_images/214945/gallery_01.webp;/upload/vvm_images/import_images/214945/gallery_02.webp;/upload/vvm_images/import_images/214945/gallery_03.webp;/upload/vvm_images/import_images/214945/gallery_04.webp;/upload/vvm_images/import_images/214945/gallery_05.webp;/upload/vvm_images/import_images/214945/gallery_06.webp;/upload/vvm_images/import_images/214945/gallery_07.webp;/upload/vvm_images/import_images/214945/gallery_08.webp;/upload/vvm_images/import_images/214945/gallery_09.webp</t>
         </is>
       </c>
     </row>
@@ -3006,11 +2630,7 @@
           <t>/upload/vvm_images/import_images/214946/preview.webp</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/214946/nan</t>
-        </is>
-      </c>
+      <c r="C152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3023,11 +2643,7 @@
           <t>/upload/vvm_images/import_images/211352/preview.webp</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/211352/nan</t>
-        </is>
-      </c>
+      <c r="C153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3040,11 +2656,7 @@
           <t>/upload/vvm_images/import_images/211353/preview.webp</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/211353/nan</t>
-        </is>
-      </c>
+      <c r="C154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3057,11 +2669,7 @@
           <t>/upload/vvm_images/import_images/210327/preview.webp</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210327/nan</t>
-        </is>
-      </c>
+      <c r="C155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3076,7 +2684,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/179473/gallery_01.webp|/upload/vvm_images/import_images/179473/gallery_02.webp|/upload/vvm_images/import_images/179473/gallery_03.webp|/upload/vvm_images/import_images/179473/gallery_04.webp|/upload/vvm_images/import_images/179473/gallery_05.webp|/upload/vvm_images/import_images/179473/gallery_06.webp|/upload/vvm_images/import_images/179473/gallery_07.webp|/upload/vvm_images/import_images/179473/gallery_08.webp|/upload/vvm_images/import_images/179473/gallery_09.webp</t>
+          <t>/upload/vvm_images/import_images/179473/gallery_01.webp;/upload/vvm_images/import_images/179473/gallery_02.webp;/upload/vvm_images/import_images/179473/gallery_03.webp;/upload/vvm_images/import_images/179473/gallery_04.webp;/upload/vvm_images/import_images/179473/gallery_05.webp;/upload/vvm_images/import_images/179473/gallery_06.webp;/upload/vvm_images/import_images/179473/gallery_07.webp;/upload/vvm_images/import_images/179473/gallery_08.webp;/upload/vvm_images/import_images/179473/gallery_09.webp</t>
         </is>
       </c>
     </row>
@@ -3093,7 +2701,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207387/gallery_01.webp|/upload/vvm_images/import_images/207387/gallery_02.webp|/upload/vvm_images/import_images/207387/gallery_03.webp|/upload/vvm_images/import_images/207387/gallery_04.webp|/upload/vvm_images/import_images/207387/gallery_05.webp|/upload/vvm_images/import_images/207387/gallery_06.webp|/upload/vvm_images/import_images/207387/gallery_07.webp|/upload/vvm_images/import_images/207387/gallery_08.webp|/upload/vvm_images/import_images/207387/gallery_09.webp|/upload/vvm_images/import_images/207387/gallery_10.webp|/upload/vvm_images/import_images/207387/gallery_11.webp|/upload/vvm_images/import_images/207387/gallery_12.webp|/upload/vvm_images/import_images/207387/gallery_13.webp</t>
+          <t>/upload/vvm_images/import_images/207387/gallery_01.webp;/upload/vvm_images/import_images/207387/gallery_02.webp;/upload/vvm_images/import_images/207387/gallery_03.webp;/upload/vvm_images/import_images/207387/gallery_04.webp;/upload/vvm_images/import_images/207387/gallery_05.webp;/upload/vvm_images/import_images/207387/gallery_06.webp;/upload/vvm_images/import_images/207387/gallery_07.webp;/upload/vvm_images/import_images/207387/gallery_08.webp;/upload/vvm_images/import_images/207387/gallery_09.webp;/upload/vvm_images/import_images/207387/gallery_10.webp;/upload/vvm_images/import_images/207387/gallery_11.webp;/upload/vvm_images/import_images/207387/gallery_12.webp;/upload/vvm_images/import_images/207387/gallery_13.webp</t>
         </is>
       </c>
     </row>
@@ -3108,11 +2716,7 @@
           <t>/upload/vvm_images/import_images/204843/preview.webp</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204843/nan</t>
-        </is>
-      </c>
+      <c r="C158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3125,11 +2729,7 @@
           <t>/upload/vvm_images/import_images/195033/preview.webp</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/195033/nan</t>
-        </is>
-      </c>
+      <c r="C159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3144,7 +2744,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/204520/gallery_01.webp|/upload/vvm_images/import_images/204520/gallery_02.webp|/upload/vvm_images/import_images/204520/gallery_03.webp|/upload/vvm_images/import_images/204520/gallery_04.webp|/upload/vvm_images/import_images/204520/gallery_05.webp|/upload/vvm_images/import_images/204520/gallery_06.webp|/upload/vvm_images/import_images/204520/gallery_07.webp|/upload/vvm_images/import_images/204520/gallery_08.webp|/upload/vvm_images/import_images/204520/gallery_09.webp|/upload/vvm_images/import_images/204520/gallery_10.webp|/upload/vvm_images/import_images/204520/gallery_11.webp|/upload/vvm_images/import_images/204520/gallery_12.webp</t>
+          <t>/upload/vvm_images/import_images/204520/gallery_01.webp;/upload/vvm_images/import_images/204520/gallery_02.webp;/upload/vvm_images/import_images/204520/gallery_03.webp;/upload/vvm_images/import_images/204520/gallery_04.webp;/upload/vvm_images/import_images/204520/gallery_05.webp;/upload/vvm_images/import_images/204520/gallery_06.webp;/upload/vvm_images/import_images/204520/gallery_07.webp;/upload/vvm_images/import_images/204520/gallery_08.webp;/upload/vvm_images/import_images/204520/gallery_09.webp;/upload/vvm_images/import_images/204520/gallery_10.webp;/upload/vvm_images/import_images/204520/gallery_11.webp;/upload/vvm_images/import_images/204520/gallery_12.webp</t>
         </is>
       </c>
     </row>
@@ -3159,11 +2759,7 @@
           <t>/upload/vvm_images/import_images/204521/preview.webp</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/204521/nan</t>
-        </is>
-      </c>
+      <c r="C161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3178,7 +2774,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205697/gallery_01.webp|/upload/vvm_images/import_images/205697/gallery_02.webp|/upload/vvm_images/import_images/205697/gallery_03.webp|/upload/vvm_images/import_images/205697/gallery_04.webp|/upload/vvm_images/import_images/205697/gallery_05.webp|/upload/vvm_images/import_images/205697/gallery_06.webp|/upload/vvm_images/import_images/205697/gallery_07.webp|/upload/vvm_images/import_images/205697/gallery_08.webp|/upload/vvm_images/import_images/205697/gallery_09.webp|/upload/vvm_images/import_images/205697/gallery_10.webp|/upload/vvm_images/import_images/205697/gallery_11.webp|/upload/vvm_images/import_images/205697/gallery_12.webp</t>
+          <t>/upload/vvm_images/import_images/205697/gallery_01.webp;/upload/vvm_images/import_images/205697/gallery_02.webp;/upload/vvm_images/import_images/205697/gallery_03.webp;/upload/vvm_images/import_images/205697/gallery_04.webp;/upload/vvm_images/import_images/205697/gallery_05.webp;/upload/vvm_images/import_images/205697/gallery_06.webp;/upload/vvm_images/import_images/205697/gallery_07.webp;/upload/vvm_images/import_images/205697/gallery_08.webp;/upload/vvm_images/import_images/205697/gallery_09.webp;/upload/vvm_images/import_images/205697/gallery_10.webp;/upload/vvm_images/import_images/205697/gallery_11.webp;/upload/vvm_images/import_images/205697/gallery_12.webp</t>
         </is>
       </c>
     </row>
@@ -3193,11 +2789,7 @@
           <t>/upload/vvm_images/import_images/201315/preview.webp</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/201315/nan</t>
-        </is>
-      </c>
+      <c r="C163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -3210,11 +2802,7 @@
           <t>/upload/vvm_images/import_images/203958/preview.webp</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/203958/nan</t>
-        </is>
-      </c>
+      <c r="C164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3227,11 +2815,7 @@
           <t>/upload/vvm_images/import_images/215181/preview.webp</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215181/nan</t>
-        </is>
-      </c>
+      <c r="C165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3244,11 +2828,7 @@
           <t>/upload/vvm_images/import_images/215182/preview.webp</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215182/nan</t>
-        </is>
-      </c>
+      <c r="C166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -3261,11 +2841,7 @@
           <t>/upload/vvm_images/import_images/215212/preview.webp</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215212/nan</t>
-        </is>
-      </c>
+      <c r="C167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3278,11 +2854,7 @@
           <t>/upload/vvm_images/import_images/215214/preview.webp</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215214/nan</t>
-        </is>
-      </c>
+      <c r="C168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -3295,11 +2867,7 @@
           <t>/upload/vvm_images/import_images/215215/preview.webp</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215215/nan</t>
-        </is>
-      </c>
+      <c r="C169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -3312,11 +2880,7 @@
           <t>/upload/vvm_images/import_images/215216/preview.webp</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215216/nan</t>
-        </is>
-      </c>
+      <c r="C170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3329,11 +2893,7 @@
           <t>/upload/vvm_images/import_images/215217/preview.webp</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215217/nan</t>
-        </is>
-      </c>
+      <c r="C171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3346,11 +2906,7 @@
           <t>/upload/vvm_images/import_images/215183/preview.webp</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215183/nan</t>
-        </is>
-      </c>
+      <c r="C172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3363,11 +2919,7 @@
           <t>/upload/vvm_images/import_images/215184/preview.webp</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215184/nan</t>
-        </is>
-      </c>
+      <c r="C173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3380,11 +2932,7 @@
           <t>/upload/vvm_images/import_images/215185/preview.webp</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215185/nan</t>
-        </is>
-      </c>
+      <c r="C174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3397,11 +2945,7 @@
           <t>/upload/vvm_images/import_images/215186/preview.webp</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215186/nan</t>
-        </is>
-      </c>
+      <c r="C175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -3414,11 +2958,7 @@
           <t>/upload/vvm_images/import_images/215187/preview.webp</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215187/nan</t>
-        </is>
-      </c>
+      <c r="C176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -3431,11 +2971,7 @@
           <t>/upload/vvm_images/import_images/215188/preview.webp</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215188/nan</t>
-        </is>
-      </c>
+      <c r="C177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -3448,11 +2984,7 @@
           <t>/upload/vvm_images/import_images/215189/preview.webp</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215189/nan</t>
-        </is>
-      </c>
+      <c r="C178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3465,11 +2997,7 @@
           <t>/upload/vvm_images/import_images/215190/preview.webp</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215190/nan</t>
-        </is>
-      </c>
+      <c r="C179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -3482,11 +3010,7 @@
           <t>/upload/vvm_images/import_images/215192/preview.webp</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215192/nan</t>
-        </is>
-      </c>
+      <c r="C180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3499,11 +3023,7 @@
           <t>/upload/vvm_images/import_images/215193/preview.webp</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215193/nan</t>
-        </is>
-      </c>
+      <c r="C181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -3516,11 +3036,7 @@
           <t>/upload/vvm_images/import_images/215194/preview.webp</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215194/nan</t>
-        </is>
-      </c>
+      <c r="C182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3533,11 +3049,7 @@
           <t>/upload/vvm_images/import_images/215195/preview.webp</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215195/nan</t>
-        </is>
-      </c>
+      <c r="C183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -3550,11 +3062,7 @@
           <t>/upload/vvm_images/import_images/215196/preview.webp</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215196/nan</t>
-        </is>
-      </c>
+      <c r="C184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3567,11 +3075,7 @@
           <t>/upload/vvm_images/import_images/215197/preview.webp</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215197/nan</t>
-        </is>
-      </c>
+      <c r="C185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3584,11 +3088,7 @@
           <t>/upload/vvm_images/import_images/215200/preview.webp</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215200/nan</t>
-        </is>
-      </c>
+      <c r="C186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -3601,11 +3101,7 @@
           <t>/upload/vvm_images/import_images/215201/preview.webp</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215201/nan</t>
-        </is>
-      </c>
+      <c r="C187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3618,11 +3114,7 @@
           <t>/upload/vvm_images/import_images/215202/preview.webp</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215202/nan</t>
-        </is>
-      </c>
+      <c r="C188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -3635,11 +3127,7 @@
           <t>/upload/vvm_images/import_images/215203/preview.webp</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215203/nan</t>
-        </is>
-      </c>
+      <c r="C189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -3652,11 +3140,7 @@
           <t>/upload/vvm_images/import_images/215204/preview.webp</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215204/nan</t>
-        </is>
-      </c>
+      <c r="C190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -3669,11 +3153,7 @@
           <t>/upload/vvm_images/import_images/215206/preview.webp</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215206/nan</t>
-        </is>
-      </c>
+      <c r="C191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -3686,11 +3166,7 @@
           <t>/upload/vvm_images/import_images/215208/preview.webp</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/215208/nan</t>
-        </is>
-      </c>
+      <c r="C192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -3703,11 +3179,7 @@
           <t>/upload/vvm_images/import_images/207367/preview.webp</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/207367/nan</t>
-        </is>
-      </c>
+      <c r="C193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -3720,11 +3192,7 @@
           <t>/upload/vvm_images/import_images/207368/preview.webp</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/207368/nan</t>
-        </is>
-      </c>
+      <c r="C194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -3737,11 +3205,7 @@
           <t>/upload/vvm_images/import_images/176460/preview.webp</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/176460/nan</t>
-        </is>
-      </c>
+      <c r="C195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3754,11 +3218,7 @@
           <t>/upload/vvm_images/import_images/205224/preview.webp</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205224/nan</t>
-        </is>
-      </c>
+      <c r="C196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -3773,7 +3233,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205225/gallery_01.webp|/upload/vvm_images/import_images/205225/gallery_02.webp|/upload/vvm_images/import_images/205225/gallery_03.webp|/upload/vvm_images/import_images/205225/gallery_04.webp|/upload/vvm_images/import_images/205225/gallery_05.webp|/upload/vvm_images/import_images/205225/gallery_06.webp|/upload/vvm_images/import_images/205225/gallery_07.webp|/upload/vvm_images/import_images/205225/gallery_08.webp|/upload/vvm_images/import_images/205225/gallery_09.webp|/upload/vvm_images/import_images/205225/gallery_10.webp|/upload/vvm_images/import_images/205225/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/205225/gallery_01.webp;/upload/vvm_images/import_images/205225/gallery_02.webp;/upload/vvm_images/import_images/205225/gallery_03.webp;/upload/vvm_images/import_images/205225/gallery_04.webp;/upload/vvm_images/import_images/205225/gallery_05.webp;/upload/vvm_images/import_images/205225/gallery_06.webp;/upload/vvm_images/import_images/205225/gallery_07.webp;/upload/vvm_images/import_images/205225/gallery_08.webp;/upload/vvm_images/import_images/205225/gallery_09.webp;/upload/vvm_images/import_images/205225/gallery_10.webp;/upload/vvm_images/import_images/205225/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3250,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205226/gallery_01.webp|/upload/vvm_images/import_images/205226/gallery_02.webp|/upload/vvm_images/import_images/205226/gallery_03.webp|/upload/vvm_images/import_images/205226/gallery_04.webp|/upload/vvm_images/import_images/205226/gallery_05.webp|/upload/vvm_images/import_images/205226/gallery_06.webp|/upload/vvm_images/import_images/205226/gallery_07.webp|/upload/vvm_images/import_images/205226/gallery_08.webp|/upload/vvm_images/import_images/205226/gallery_09.webp|/upload/vvm_images/import_images/205226/gallery_10.webp|/upload/vvm_images/import_images/205226/gallery_11.webp|/upload/vvm_images/import_images/205226/gallery_12.webp</t>
+          <t>/upload/vvm_images/import_images/205226/gallery_01.webp;/upload/vvm_images/import_images/205226/gallery_02.webp;/upload/vvm_images/import_images/205226/gallery_03.webp;/upload/vvm_images/import_images/205226/gallery_04.webp;/upload/vvm_images/import_images/205226/gallery_05.webp;/upload/vvm_images/import_images/205226/gallery_06.webp;/upload/vvm_images/import_images/205226/gallery_07.webp;/upload/vvm_images/import_images/205226/gallery_08.webp;/upload/vvm_images/import_images/205226/gallery_09.webp;/upload/vvm_images/import_images/205226/gallery_10.webp;/upload/vvm_images/import_images/205226/gallery_11.webp;/upload/vvm_images/import_images/205226/gallery_12.webp</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3267,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/205228/gallery_01.webp|/upload/vvm_images/import_images/205228/gallery_02.webp|/upload/vvm_images/import_images/205228/gallery_03.webp|/upload/vvm_images/import_images/205228/gallery_04.webp|/upload/vvm_images/import_images/205228/gallery_05.webp|/upload/vvm_images/import_images/205228/gallery_06.webp|/upload/vvm_images/import_images/205228/gallery_07.webp|/upload/vvm_images/import_images/205228/gallery_08.webp|/upload/vvm_images/import_images/205228/gallery_09.webp|/upload/vvm_images/import_images/205228/gallery_10.webp|/upload/vvm_images/import_images/205228/gallery_11.webp</t>
+          <t>/upload/vvm_images/import_images/205228/gallery_01.webp;/upload/vvm_images/import_images/205228/gallery_02.webp;/upload/vvm_images/import_images/205228/gallery_03.webp;/upload/vvm_images/import_images/205228/gallery_04.webp;/upload/vvm_images/import_images/205228/gallery_05.webp;/upload/vvm_images/import_images/205228/gallery_06.webp;/upload/vvm_images/import_images/205228/gallery_07.webp;/upload/vvm_images/import_images/205228/gallery_08.webp;/upload/vvm_images/import_images/205228/gallery_09.webp;/upload/vvm_images/import_images/205228/gallery_10.webp;/upload/vvm_images/import_images/205228/gallery_11.webp</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3284,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/206452/gallery_01.webp|/upload/vvm_images/import_images/206452/gallery_02.webp|/upload/vvm_images/import_images/206452/gallery_03.webp|/upload/vvm_images/import_images/206452/gallery_04.webp|/upload/vvm_images/import_images/206452/gallery_05.webp|/upload/vvm_images/import_images/206452/gallery_06.webp|/upload/vvm_images/import_images/206452/gallery_07.webp|/upload/vvm_images/import_images/206452/gallery_08.webp|/upload/vvm_images/import_images/206452/gallery_09.webp|/upload/vvm_images/import_images/206452/gallery_10.webp|/upload/vvm_images/import_images/206452/gallery_11.webp|/upload/vvm_images/import_images/206452/gallery_12.webp|/upload/vvm_images/import_images/206452/gallery_13.webp|/upload/vvm_images/import_images/206452/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/206452/gallery_01.webp;/upload/vvm_images/import_images/206452/gallery_02.webp;/upload/vvm_images/import_images/206452/gallery_03.webp;/upload/vvm_images/import_images/206452/gallery_04.webp;/upload/vvm_images/import_images/206452/gallery_05.webp;/upload/vvm_images/import_images/206452/gallery_06.webp;/upload/vvm_images/import_images/206452/gallery_07.webp;/upload/vvm_images/import_images/206452/gallery_08.webp;/upload/vvm_images/import_images/206452/gallery_09.webp;/upload/vvm_images/import_images/206452/gallery_10.webp;/upload/vvm_images/import_images/206452/gallery_11.webp;/upload/vvm_images/import_images/206452/gallery_12.webp;/upload/vvm_images/import_images/206452/gallery_13.webp;/upload/vvm_images/import_images/206452/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3301,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207405/gallery_01.webp|/upload/vvm_images/import_images/207405/gallery_02.webp|/upload/vvm_images/import_images/207405/gallery_03.webp|/upload/vvm_images/import_images/207405/gallery_04.webp|/upload/vvm_images/import_images/207405/gallery_05.webp|/upload/vvm_images/import_images/207405/gallery_06.webp|/upload/vvm_images/import_images/207405/gallery_07.webp|/upload/vvm_images/import_images/207405/gallery_08.webp|/upload/vvm_images/import_images/207405/gallery_09.webp|/upload/vvm_images/import_images/207405/gallery_10.webp|/upload/vvm_images/import_images/207405/gallery_11.webp|/upload/vvm_images/import_images/207405/gallery_12.webp|/upload/vvm_images/import_images/207405/gallery_13.webp|/upload/vvm_images/import_images/207405/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/207405/gallery_01.webp;/upload/vvm_images/import_images/207405/gallery_02.webp;/upload/vvm_images/import_images/207405/gallery_03.webp;/upload/vvm_images/import_images/207405/gallery_04.webp;/upload/vvm_images/import_images/207405/gallery_05.webp;/upload/vvm_images/import_images/207405/gallery_06.webp;/upload/vvm_images/import_images/207405/gallery_07.webp;/upload/vvm_images/import_images/207405/gallery_08.webp;/upload/vvm_images/import_images/207405/gallery_09.webp;/upload/vvm_images/import_images/207405/gallery_10.webp;/upload/vvm_images/import_images/207405/gallery_11.webp;/upload/vvm_images/import_images/207405/gallery_12.webp;/upload/vvm_images/import_images/207405/gallery_13.webp;/upload/vvm_images/import_images/207405/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -3858,7 +3318,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207388/gallery_01.webp|/upload/vvm_images/import_images/207388/gallery_02.webp|/upload/vvm_images/import_images/207388/gallery_03.webp|/upload/vvm_images/import_images/207388/gallery_04.webp|/upload/vvm_images/import_images/207388/gallery_05.webp|/upload/vvm_images/import_images/207388/gallery_06.webp|/upload/vvm_images/import_images/207388/gallery_07.webp|/upload/vvm_images/import_images/207388/gallery_08.webp|/upload/vvm_images/import_images/207388/gallery_09.webp|/upload/vvm_images/import_images/207388/gallery_10.webp|/upload/vvm_images/import_images/207388/gallery_11.webp|/upload/vvm_images/import_images/207388/gallery_12.webp|/upload/vvm_images/import_images/207388/gallery_13.webp|/upload/vvm_images/import_images/207388/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/207388/gallery_01.webp;/upload/vvm_images/import_images/207388/gallery_02.webp;/upload/vvm_images/import_images/207388/gallery_03.webp;/upload/vvm_images/import_images/207388/gallery_04.webp;/upload/vvm_images/import_images/207388/gallery_05.webp;/upload/vvm_images/import_images/207388/gallery_06.webp;/upload/vvm_images/import_images/207388/gallery_07.webp;/upload/vvm_images/import_images/207388/gallery_08.webp;/upload/vvm_images/import_images/207388/gallery_09.webp;/upload/vvm_images/import_images/207388/gallery_10.webp;/upload/vvm_images/import_images/207388/gallery_11.webp;/upload/vvm_images/import_images/207388/gallery_12.webp;/upload/vvm_images/import_images/207388/gallery_13.webp;/upload/vvm_images/import_images/207388/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3335,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207393/gallery_01.webp|/upload/vvm_images/import_images/207393/gallery_02.webp|/upload/vvm_images/import_images/207393/gallery_03.webp|/upload/vvm_images/import_images/207393/gallery_04.webp|/upload/vvm_images/import_images/207393/gallery_05.webp|/upload/vvm_images/import_images/207393/gallery_06.webp|/upload/vvm_images/import_images/207393/gallery_07.webp|/upload/vvm_images/import_images/207393/gallery_08.webp|/upload/vvm_images/import_images/207393/gallery_09.webp|/upload/vvm_images/import_images/207393/gallery_10.webp|/upload/vvm_images/import_images/207393/gallery_11.webp|/upload/vvm_images/import_images/207393/gallery_12.webp|/upload/vvm_images/import_images/207393/gallery_13.webp|/upload/vvm_images/import_images/207393/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/207393/gallery_01.webp;/upload/vvm_images/import_images/207393/gallery_02.webp;/upload/vvm_images/import_images/207393/gallery_03.webp;/upload/vvm_images/import_images/207393/gallery_04.webp;/upload/vvm_images/import_images/207393/gallery_05.webp;/upload/vvm_images/import_images/207393/gallery_06.webp;/upload/vvm_images/import_images/207393/gallery_07.webp;/upload/vvm_images/import_images/207393/gallery_08.webp;/upload/vvm_images/import_images/207393/gallery_09.webp;/upload/vvm_images/import_images/207393/gallery_10.webp;/upload/vvm_images/import_images/207393/gallery_11.webp;/upload/vvm_images/import_images/207393/gallery_12.webp;/upload/vvm_images/import_images/207393/gallery_13.webp;/upload/vvm_images/import_images/207393/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -3890,11 +3350,7 @@
           <t>/upload/vvm_images/import_images/210344/preview.webp</t>
         </is>
       </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210344/nan</t>
-        </is>
-      </c>
+      <c r="C204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -3907,11 +3363,7 @@
           <t>/upload/vvm_images/import_images/TAP12509-2/preview.webp</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TAP12509-2/nan</t>
-        </is>
-      </c>
+      <c r="C205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -3924,11 +3376,7 @@
           <t>/upload/vvm_images/import_images/TAP15010-1/preview.webp</t>
         </is>
       </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TAP15010-1/nan</t>
-        </is>
-      </c>
+      <c r="C206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -3941,11 +3389,7 @@
           <t>/upload/vvm_images/import_images/195517/preview.webp</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/195517/nan</t>
-        </is>
-      </c>
+      <c r="C207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -3958,11 +3402,7 @@
           <t>/upload/vvm_images/import_images/195518/preview.webp</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/195518/nan</t>
-        </is>
-      </c>
+      <c r="C208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -3975,11 +3415,7 @@
           <t>/upload/vvm_images/import_images/TV70L-29/preview.webp</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TV70L-29/nan</t>
-        </is>
-      </c>
+      <c r="C209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -3992,11 +3428,7 @@
           <t>/upload/vvm_images/import_images/188620/preview.webp</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/188620/nan</t>
-        </is>
-      </c>
+      <c r="C210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -4009,11 +3441,7 @@
           <t>/upload/vvm_images/import_images/210192/preview.webp</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210192/nan</t>
-        </is>
-      </c>
+      <c r="C211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -4026,11 +3454,7 @@
           <t>/upload/vvm_images/import_images/TV20L-18/preview.webp</t>
         </is>
       </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TV20L-18/nan</t>
-        </is>
-      </c>
+      <c r="C212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -4043,11 +3467,7 @@
           <t>/upload/vvm_images/import_images/TV30L-C-38/preview.webp</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TV30L-C-38/nan</t>
-        </is>
-      </c>
+      <c r="C213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -4060,11 +3480,7 @@
           <t>/upload/vvm_images/import_images/TV20L-36/preview.webp</t>
         </is>
       </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TV20L-36/nan</t>
-        </is>
-      </c>
+      <c r="C214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -4079,7 +3495,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/206083/gallery_01.webp|/upload/vvm_images/import_images/206083/gallery_02.webp|/upload/vvm_images/import_images/206083/gallery_03.webp|/upload/vvm_images/import_images/206083/gallery_04.webp|/upload/vvm_images/import_images/206083/gallery_05.webp</t>
+          <t>/upload/vvm_images/import_images/206083/gallery_01.webp;/upload/vvm_images/import_images/206083/gallery_02.webp;/upload/vvm_images/import_images/206083/gallery_03.webp;/upload/vvm_images/import_images/206083/gallery_04.webp;/upload/vvm_images/import_images/206083/gallery_05.webp</t>
         </is>
       </c>
     </row>
@@ -4094,11 +3510,7 @@
           <t>/upload/vvm_images/import_images/TS21509-1/preview.webp</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TS21509-1/nan</t>
-        </is>
-      </c>
+      <c r="C216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -4111,11 +3523,7 @@
           <t>/upload/vvm_images/import_images/TS22513-2/preview.webp</t>
         </is>
       </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/TS22513-2/nan</t>
-        </is>
-      </c>
+      <c r="C217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -4128,11 +3536,7 @@
           <t>/upload/vvm_images/import_images/207378/preview.webp</t>
         </is>
       </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/207378/nan</t>
-        </is>
-      </c>
+      <c r="C218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -4147,7 +3551,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210314/gallery_01.webp|/upload/vvm_images/import_images/210314/gallery_02.webp|/upload/vvm_images/import_images/210314/gallery_03.webp|/upload/vvm_images/import_images/210314/gallery_04.webp|/upload/vvm_images/import_images/210314/gallery_05.webp|/upload/vvm_images/import_images/210314/gallery_06.webp|/upload/vvm_images/import_images/210314/gallery_07.webp|/upload/vvm_images/import_images/210314/gallery_08.webp|/upload/vvm_images/import_images/210314/gallery_09.webp|/upload/vvm_images/import_images/210314/gallery_10.webp|/upload/vvm_images/import_images/210314/gallery_11.webp|/upload/vvm_images/import_images/210314/gallery_12.webp</t>
+          <t>/upload/vvm_images/import_images/210314/gallery_01.webp;/upload/vvm_images/import_images/210314/gallery_02.webp;/upload/vvm_images/import_images/210314/gallery_03.webp;/upload/vvm_images/import_images/210314/gallery_04.webp;/upload/vvm_images/import_images/210314/gallery_05.webp;/upload/vvm_images/import_images/210314/gallery_06.webp;/upload/vvm_images/import_images/210314/gallery_07.webp;/upload/vvm_images/import_images/210314/gallery_08.webp;/upload/vvm_images/import_images/210314/gallery_09.webp;/upload/vvm_images/import_images/210314/gallery_10.webp;/upload/vvm_images/import_images/210314/gallery_11.webp;/upload/vvm_images/import_images/210314/gallery_12.webp</t>
         </is>
       </c>
     </row>
@@ -4164,7 +3568,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210315/gallery_01.webp|/upload/vvm_images/import_images/210315/gallery_02.webp|/upload/vvm_images/import_images/210315/gallery_03.webp|/upload/vvm_images/import_images/210315/gallery_04.webp|/upload/vvm_images/import_images/210315/gallery_05.webp|/upload/vvm_images/import_images/210315/gallery_06.webp|/upload/vvm_images/import_images/210315/gallery_07.webp|/upload/vvm_images/import_images/210315/gallery_08.webp|/upload/vvm_images/import_images/210315/gallery_09.webp|/upload/vvm_images/import_images/210315/gallery_10.webp|/upload/vvm_images/import_images/210315/gallery_11.webp|/upload/vvm_images/import_images/210315/gallery_12.webp|/upload/vvm_images/import_images/210315/gallery_13.webp|/upload/vvm_images/import_images/210315/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/210315/gallery_01.webp;/upload/vvm_images/import_images/210315/gallery_02.webp;/upload/vvm_images/import_images/210315/gallery_03.webp;/upload/vvm_images/import_images/210315/gallery_04.webp;/upload/vvm_images/import_images/210315/gallery_05.webp;/upload/vvm_images/import_images/210315/gallery_06.webp;/upload/vvm_images/import_images/210315/gallery_07.webp;/upload/vvm_images/import_images/210315/gallery_08.webp;/upload/vvm_images/import_images/210315/gallery_09.webp;/upload/vvm_images/import_images/210315/gallery_10.webp;/upload/vvm_images/import_images/210315/gallery_11.webp;/upload/vvm_images/import_images/210315/gallery_12.webp;/upload/vvm_images/import_images/210315/gallery_13.webp;/upload/vvm_images/import_images/210315/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -4181,7 +3585,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210316/gallery_01.webp|/upload/vvm_images/import_images/210316/gallery_02.webp|/upload/vvm_images/import_images/210316/gallery_03.webp|/upload/vvm_images/import_images/210316/gallery_04.webp|/upload/vvm_images/import_images/210316/gallery_05.webp|/upload/vvm_images/import_images/210316/gallery_06.webp|/upload/vvm_images/import_images/210316/gallery_07.webp|/upload/vvm_images/import_images/210316/gallery_08.webp|/upload/vvm_images/import_images/210316/gallery_09.webp|/upload/vvm_images/import_images/210316/gallery_10.webp|/upload/vvm_images/import_images/210316/gallery_11.webp|/upload/vvm_images/import_images/210316/gallery_12.webp|/upload/vvm_images/import_images/210316/gallery_13.webp|/upload/vvm_images/import_images/210316/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/210316/gallery_01.webp;/upload/vvm_images/import_images/210316/gallery_02.webp;/upload/vvm_images/import_images/210316/gallery_03.webp;/upload/vvm_images/import_images/210316/gallery_04.webp;/upload/vvm_images/import_images/210316/gallery_05.webp;/upload/vvm_images/import_images/210316/gallery_06.webp;/upload/vvm_images/import_images/210316/gallery_07.webp;/upload/vvm_images/import_images/210316/gallery_08.webp;/upload/vvm_images/import_images/210316/gallery_09.webp;/upload/vvm_images/import_images/210316/gallery_10.webp;/upload/vvm_images/import_images/210316/gallery_11.webp;/upload/vvm_images/import_images/210316/gallery_12.webp;/upload/vvm_images/import_images/210316/gallery_13.webp;/upload/vvm_images/import_images/210316/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -4198,7 +3602,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210317/gallery_01.webp|/upload/vvm_images/import_images/210317/gallery_02.webp|/upload/vvm_images/import_images/210317/gallery_03.webp|/upload/vvm_images/import_images/210317/gallery_04.webp|/upload/vvm_images/import_images/210317/gallery_05.webp|/upload/vvm_images/import_images/210317/gallery_06.webp|/upload/vvm_images/import_images/210317/gallery_07.webp|/upload/vvm_images/import_images/210317/gallery_08.webp|/upload/vvm_images/import_images/210317/gallery_09.webp|/upload/vvm_images/import_images/210317/gallery_10.webp|/upload/vvm_images/import_images/210317/gallery_11.webp|/upload/vvm_images/import_images/210317/gallery_12.webp</t>
+          <t>/upload/vvm_images/import_images/210317/gallery_01.webp;/upload/vvm_images/import_images/210317/gallery_02.webp;/upload/vvm_images/import_images/210317/gallery_03.webp;/upload/vvm_images/import_images/210317/gallery_04.webp;/upload/vvm_images/import_images/210317/gallery_05.webp;/upload/vvm_images/import_images/210317/gallery_06.webp;/upload/vvm_images/import_images/210317/gallery_07.webp;/upload/vvm_images/import_images/210317/gallery_08.webp;/upload/vvm_images/import_images/210317/gallery_09.webp;/upload/vvm_images/import_images/210317/gallery_10.webp;/upload/vvm_images/import_images/210317/gallery_11.webp;/upload/vvm_images/import_images/210317/gallery_12.webp</t>
         </is>
       </c>
     </row>
@@ -4215,7 +3619,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210318/gallery_01.webp|/upload/vvm_images/import_images/210318/gallery_02.webp|/upload/vvm_images/import_images/210318/gallery_03.webp|/upload/vvm_images/import_images/210318/gallery_04.webp|/upload/vvm_images/import_images/210318/gallery_05.webp|/upload/vvm_images/import_images/210318/gallery_06.webp|/upload/vvm_images/import_images/210318/gallery_07.webp|/upload/vvm_images/import_images/210318/gallery_08.webp|/upload/vvm_images/import_images/210318/gallery_09.webp|/upload/vvm_images/import_images/210318/gallery_10.webp|/upload/vvm_images/import_images/210318/gallery_11.webp|/upload/vvm_images/import_images/210318/gallery_12.webp|/upload/vvm_images/import_images/210318/gallery_13.webp|/upload/vvm_images/import_images/210318/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/210318/gallery_01.webp;/upload/vvm_images/import_images/210318/gallery_02.webp;/upload/vvm_images/import_images/210318/gallery_03.webp;/upload/vvm_images/import_images/210318/gallery_04.webp;/upload/vvm_images/import_images/210318/gallery_05.webp;/upload/vvm_images/import_images/210318/gallery_06.webp;/upload/vvm_images/import_images/210318/gallery_07.webp;/upload/vvm_images/import_images/210318/gallery_08.webp;/upload/vvm_images/import_images/210318/gallery_09.webp;/upload/vvm_images/import_images/210318/gallery_10.webp;/upload/vvm_images/import_images/210318/gallery_11.webp;/upload/vvm_images/import_images/210318/gallery_12.webp;/upload/vvm_images/import_images/210318/gallery_13.webp;/upload/vvm_images/import_images/210318/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -4232,7 +3636,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/210319/gallery_01.webp|/upload/vvm_images/import_images/210319/gallery_02.webp|/upload/vvm_images/import_images/210319/gallery_03.webp|/upload/vvm_images/import_images/210319/gallery_04.webp|/upload/vvm_images/import_images/210319/gallery_05.webp|/upload/vvm_images/import_images/210319/gallery_06.webp|/upload/vvm_images/import_images/210319/gallery_07.webp|/upload/vvm_images/import_images/210319/gallery_08.webp|/upload/vvm_images/import_images/210319/gallery_09.webp|/upload/vvm_images/import_images/210319/gallery_10.webp|/upload/vvm_images/import_images/210319/gallery_11.webp|/upload/vvm_images/import_images/210319/gallery_12.webp|/upload/vvm_images/import_images/210319/gallery_13.webp|/upload/vvm_images/import_images/210319/gallery_14.webp</t>
+          <t>/upload/vvm_images/import_images/210319/gallery_01.webp;/upload/vvm_images/import_images/210319/gallery_02.webp;/upload/vvm_images/import_images/210319/gallery_03.webp;/upload/vvm_images/import_images/210319/gallery_04.webp;/upload/vvm_images/import_images/210319/gallery_05.webp;/upload/vvm_images/import_images/210319/gallery_06.webp;/upload/vvm_images/import_images/210319/gallery_07.webp;/upload/vvm_images/import_images/210319/gallery_08.webp;/upload/vvm_images/import_images/210319/gallery_09.webp;/upload/vvm_images/import_images/210319/gallery_10.webp;/upload/vvm_images/import_images/210319/gallery_11.webp;/upload/vvm_images/import_images/210319/gallery_12.webp;/upload/vvm_images/import_images/210319/gallery_13.webp;/upload/vvm_images/import_images/210319/gallery_14.webp</t>
         </is>
       </c>
     </row>
@@ -4249,7 +3653,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/207374/gallery_01.webp|/upload/vvm_images/import_images/207374/gallery_02.webp|/upload/vvm_images/import_images/207374/gallery_03.webp|/upload/vvm_images/import_images/207374/gallery_04.webp|/upload/vvm_images/import_images/207374/gallery_05.webp|/upload/vvm_images/import_images/207374/gallery_06.webp|/upload/vvm_images/import_images/207374/gallery_07.webp|/upload/vvm_images/import_images/207374/gallery_08.webp|/upload/vvm_images/import_images/207374/gallery_09.webp|/upload/vvm_images/import_images/207374/gallery_10.webp</t>
+          <t>/upload/vvm_images/import_images/207374/gallery_01.webp;/upload/vvm_images/import_images/207374/gallery_02.webp;/upload/vvm_images/import_images/207374/gallery_03.webp;/upload/vvm_images/import_images/207374/gallery_04.webp;/upload/vvm_images/import_images/207374/gallery_05.webp;/upload/vvm_images/import_images/207374/gallery_06.webp;/upload/vvm_images/import_images/207374/gallery_07.webp;/upload/vvm_images/import_images/207374/gallery_08.webp;/upload/vvm_images/import_images/207374/gallery_09.webp;/upload/vvm_images/import_images/207374/gallery_10.webp</t>
         </is>
       </c>
     </row>
@@ -4264,11 +3668,7 @@
           <t>/upload/vvm_images/import_images/210866/preview.webp</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210866/nan</t>
-        </is>
-      </c>
+      <c r="C226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -4281,11 +3681,7 @@
           <t>/upload/vvm_images/import_images/210867/preview.webp</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/210867/nan</t>
-        </is>
-      </c>
+      <c r="C227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -4300,7 +3696,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/LPS508-01/gallery_01.webp|/upload/vvm_images/import_images/LPS508-01/gallery_02.webp|/upload/vvm_images/import_images/LPS508-01/gallery_03.webp|/upload/vvm_images/import_images/LPS508-01/gallery_04.webp|/upload/vvm_images/import_images/LPS508-01/gallery_05.webp|/upload/vvm_images/import_images/LPS508-01/gallery_06.webp|/upload/vvm_images/import_images/LPS508-01/gallery_07.webp|/upload/vvm_images/import_images/LPS508-01/gallery_08.webp|/upload/vvm_images/import_images/LPS508-01/gallery_09.webp|/upload/vvm_images/import_images/LPS508-01/gallery_10.webp</t>
+          <t>/upload/vvm_images/import_images/LPS508-01/gallery_01.webp;/upload/vvm_images/import_images/LPS508-01/gallery_02.webp;/upload/vvm_images/import_images/LPS508-01/gallery_03.webp;/upload/vvm_images/import_images/LPS508-01/gallery_04.webp;/upload/vvm_images/import_images/LPS508-01/gallery_05.webp;/upload/vvm_images/import_images/LPS508-01/gallery_06.webp;/upload/vvm_images/import_images/LPS508-01/gallery_07.webp;/upload/vvm_images/import_images/LPS508-01/gallery_08.webp;/upload/vvm_images/import_images/LPS508-01/gallery_09.webp;/upload/vvm_images/import_images/LPS508-01/gallery_10.webp</t>
         </is>
       </c>
     </row>
@@ -4315,11 +3711,7 @@
           <t>/upload/vvm_images/import_images/188617/preview.webp</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/188617/nan</t>
-        </is>
-      </c>
+      <c r="C229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4334,7 +3726,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/214190/gallery_01.webp|/upload/vvm_images/import_images/214190/gallery_02.webp</t>
+          <t>/upload/vvm_images/import_images/214190/gallery_01.webp;/upload/vvm_images/import_images/214190/gallery_02.webp</t>
         </is>
       </c>
     </row>
@@ -4351,7 +3743,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>/upload/vvm_images/import_images/214191/gallery_01.webp|/upload/vvm_images/import_images/214191/gallery_02.webp</t>
+          <t>/upload/vvm_images/import_images/214191/gallery_01.webp;/upload/vvm_images/import_images/214191/gallery_02.webp</t>
         </is>
       </c>
     </row>
@@ -4366,11 +3758,7 @@
           <t>/upload/vvm_images/import_images/205055/preview.webp</t>
         </is>
       </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205055/nan</t>
-        </is>
-      </c>
+      <c r="C232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4383,11 +3771,7 @@
           <t>/upload/vvm_images/import_images/205054/preview.webp</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/205054/nan</t>
-        </is>
-      </c>
+      <c r="C233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -4400,11 +3784,7 @@
           <t>/upload/vvm_images/import_images/191893/preview.webp</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/191893/nan</t>
-        </is>
-      </c>
+      <c r="C234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -4417,11 +3797,7 @@
           <t>/upload/vvm_images/import_images/191897/preview.webp</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>/upload/vvm_images/import_images/191897/nan</t>
-        </is>
-      </c>
+      <c r="C235" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>